<commit_message>
reshuffled for correct samples
</commit_message>
<xml_diff>
--- a/p/content_by_grammar.xlsx
+++ b/p/content_by_grammar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adsv\private\books\language\ingush\Dahkilgov\github\dahkilgov\p\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{019E691F-AD27-4281-A572-6625E48647D1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{F7F74362-DD83-4FE1-8264-EF9D009903B1}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2415" windowWidth="38640" windowHeight="21120" xr2:uid="{AC639D1C-64A7-45F6-9CFA-A1A688E9895B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="732" uniqueCount="312">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="733" uniqueCount="313">
   <si>
     <t>Причастие, несамостоятельное, настоящее время</t>
   </si>
@@ -170,9 +170,6 @@
     <t>Глагол, времена, будущее возможное время.</t>
   </si>
   <si>
-    <t>Глагол, вопросительно-отрицательный оборот.</t>
-  </si>
-  <si>
     <t>Существительное, суффиксы для абстрактных понятий.</t>
   </si>
   <si>
@@ -293,9 +290,6 @@
     <t>Глагол, времена, давно прошедшее время.</t>
   </si>
   <si>
-    <t>Глагол, формы глаголы “быть” – “хила”.</t>
-  </si>
-  <si>
     <t>Глагол, времена, прошедшее совершенное время, отрицание с частицей -вац.</t>
   </si>
   <si>
@@ -975,6 +969,15 @@
   </si>
   <si>
     <t>Глагол, наклонение, условное.</t>
+  </si>
+  <si>
+    <t>103</t>
+  </si>
+  <si>
+    <t>Глагол, формы глагола "да" - делать.</t>
+  </si>
+  <si>
+    <t>Глагол, формы глагола "хила" - “быть”.</t>
   </si>
 </sst>
 </file>
@@ -1385,46 +1388,47 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{1CF10F6C-6A1D-4B85-A089-8B107B77E54C}">
-  <dimension ref="A1:E171"/>
+  <dimension ref="A1:F171"/>
   <sheetFormatPr defaultRowHeight="14.4" x14ac:dyDescent="0.3"/>
   <cols>
     <col min="1" max="1" width="8.88671875" style="4"/>
     <col min="2" max="2" width="93" style="2" bestFit="1" customWidth="1"/>
     <col min="3" max="4" width="8.88671875" style="3"/>
+    <col min="6" max="6" width="24.77734375" customWidth="1"/>
   </cols>
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1432,16 +1436,16 @@
         <v>144</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1449,50 +1453,50 @@
         <v>105</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>276</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>159</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>278</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>161</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>141</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>280</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>116</v>
+        <v>114</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1500,33 +1504,33 @@
         <v>152</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E7" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E8" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1534,84 +1538,84 @@
         <v>166</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E9" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E10" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E11" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>184</v>
+        <v>182</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>135</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>137</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>139</v>
-      </c>
       <c r="E12" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>185</v>
+        <v>183</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E13" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -1619,16 +1623,16 @@
         <v>124</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E14" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1636,16 +1640,16 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E15" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -1653,135 +1657,135 @@
         <v>128</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E16" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>186</v>
+        <v>184</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>129</v>
+        <v>127</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E17" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>187</v>
+        <v>185</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E18" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>188</v>
+        <v>186</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E19" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E20" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E21" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E22" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="B23" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E23" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
@@ -1789,33 +1793,33 @@
         <v>160</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>90</v>
+        <v>88</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E24" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E25" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
@@ -1823,16 +1827,16 @@
         <v>165</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>111</v>
+        <v>109</v>
       </c>
       <c r="C26" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D26" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="E26" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
@@ -1840,50 +1844,50 @@
         <v>137</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E27" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E28" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E29" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
@@ -1891,16 +1895,16 @@
         <v>138</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E30" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
@@ -1908,33 +1912,33 @@
         <v>117</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E31" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E32" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1942,67 +1946,67 @@
         <v>147</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E33" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E34" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E35" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="B36" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E36" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
@@ -2010,67 +2014,67 @@
         <v>114</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>47</v>
+        <v>46</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E37" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E38" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="B39" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E39" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E40" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
@@ -2078,16 +2082,16 @@
         <v>134</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C41" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D41" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D41" s="3" t="s">
-        <v>143</v>
-      </c>
       <c r="E41" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
@@ -2095,152 +2099,152 @@
         <v>106</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E42" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E43" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E44" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="B45" s="1" t="s">
         <v>36</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E45" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E46" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="B47" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E47" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E48" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="B49" s="1" t="s">
         <v>35</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E49" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E50" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
@@ -2248,16 +2252,16 @@
         <v>141</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E51" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
@@ -2265,16 +2269,16 @@
         <v>167</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>91</v>
+        <v>89</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E52" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
@@ -2282,16 +2286,16 @@
         <v>155</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>86</v>
+        <v>84</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E53" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -2299,16 +2303,16 @@
         <v>170</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>92</v>
+        <v>90</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E54" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
@@ -2316,101 +2320,101 @@
         <v>154</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>103</v>
+        <v>101</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E55" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E56" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E57" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E58" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>166</v>
+        <v>164</v>
       </c>
       <c r="E59" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>167</v>
+        <v>165</v>
       </c>
       <c r="E60" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
@@ -2418,16 +2422,16 @@
         <v>100</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>168</v>
+        <v>166</v>
       </c>
       <c r="E61" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
@@ -2435,101 +2439,101 @@
         <v>101</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="E62" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>294</v>
+        <v>248</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>164</v>
+        <v>162</v>
       </c>
       <c r="E63" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="E64" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="65" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E65" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="66" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="B66" s="1" t="s">
         <v>39</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E66" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="67" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="B67" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E67" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="68" spans="1:5" x14ac:dyDescent="0.3">
@@ -2537,33 +2541,33 @@
         <v>142</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E68" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="69" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>297</v>
+        <v>295</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E69" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="70" spans="1:5" x14ac:dyDescent="0.3">
@@ -2571,50 +2575,50 @@
         <v>126</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E70" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="71" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="B71" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E71" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="72" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="B72" s="1" t="s">
-        <v>298</v>
+        <v>296</v>
       </c>
       <c r="C72" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D72" s="3" t="s">
         <v>142</v>
       </c>
-      <c r="D72" s="3" t="s">
-        <v>144</v>
-      </c>
       <c r="E72" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="73" spans="1:5" x14ac:dyDescent="0.3">
@@ -2622,33 +2626,33 @@
         <v>151</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E73" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="74" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="B74" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C74" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D74" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E74" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="75" spans="1:5" x14ac:dyDescent="0.3">
@@ -2659,30 +2663,30 @@
         <v>6</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="E75" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="76" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E76" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="77" spans="1:5" x14ac:dyDescent="0.3">
@@ -2690,16 +2694,16 @@
         <v>107</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>300</v>
+        <v>298</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E77" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="78" spans="1:5" x14ac:dyDescent="0.3">
@@ -2707,33 +2711,33 @@
         <v>164</v>
       </c>
       <c r="B78" s="1" t="s">
-        <v>301</v>
+        <v>299</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E78" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="79" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E79" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="80" spans="1:5" x14ac:dyDescent="0.3">
@@ -2741,135 +2745,135 @@
         <v>111</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>299</v>
+        <v>297</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E80" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E81" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E82" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E83" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E84" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>229</v>
+        <v>227</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E85" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>230</v>
+        <v>292</v>
       </c>
       <c r="B86" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E86" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>231</v>
+        <v>229</v>
       </c>
       <c r="B87" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E87" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
@@ -2877,16 +2881,16 @@
         <v>158</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>89</v>
+        <v>87</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E88" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
@@ -2894,16 +2898,16 @@
         <v>140</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E89" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
@@ -2914,30 +2918,30 @@
         <v>5</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
       <c r="E90" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>232</v>
+        <v>230</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>37</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="E91" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="92" spans="1:5" x14ac:dyDescent="0.3">
@@ -2945,50 +2949,50 @@
         <v>131</v>
       </c>
       <c r="B92" s="1" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="E92" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>233</v>
+        <v>231</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>94</v>
+        <v>92</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E93" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>234</v>
+        <v>232</v>
       </c>
       <c r="B94" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E94" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
@@ -2996,33 +3000,33 @@
         <v>108</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>98</v>
+        <v>96</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
       <c r="E95" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>235</v>
+        <v>233</v>
       </c>
       <c r="B96" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E96" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="97" spans="1:5" x14ac:dyDescent="0.3">
@@ -3030,67 +3034,67 @@
         <v>110</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>45</v>
+        <v>44</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="E97" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="98" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>236</v>
+        <v>234</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>53</v>
+        <v>52</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="E98" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="99" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>237</v>
+        <v>235</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="E99" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="100" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A100" s="4" t="s">
-        <v>238</v>
+        <v>236</v>
       </c>
       <c r="B100" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C100" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D100" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="D100" s="3" t="s">
-        <v>147</v>
-      </c>
       <c r="E100" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="101" spans="1:5" x14ac:dyDescent="0.3">
@@ -3098,33 +3102,33 @@
         <v>168</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>93</v>
+        <v>91</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="E101" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="102" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>239</v>
+        <v>237</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>54</v>
+        <v>53</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="E102" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="103" spans="1:5" x14ac:dyDescent="0.3">
@@ -3132,67 +3136,67 @@
         <v>104</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>99</v>
+        <v>97</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="E103" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="104" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A104" s="4" t="s">
-        <v>241</v>
+        <v>239</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>52</v>
+        <v>51</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="E104" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="105" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A105" s="4" t="s">
-        <v>240</v>
+        <v>238</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>100</v>
+        <v>98</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="E105" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="106" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A106" s="4" t="s">
-        <v>242</v>
+        <v>240</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>59</v>
+        <v>58</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E106" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="107" spans="1:5" x14ac:dyDescent="0.3">
@@ -3200,16 +3204,16 @@
         <v>153</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>85</v>
+        <v>83</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>154</v>
+        <v>152</v>
       </c>
       <c r="E107" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="108" spans="1:5" x14ac:dyDescent="0.3">
@@ -3217,16 +3221,16 @@
         <v>146</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>155</v>
+        <v>153</v>
       </c>
       <c r="E108" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="109" spans="1:5" x14ac:dyDescent="0.3">
@@ -3234,16 +3238,16 @@
         <v>115</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>97</v>
+        <v>95</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>156</v>
+        <v>154</v>
       </c>
       <c r="E109" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="110" spans="1:5" x14ac:dyDescent="0.3">
@@ -3251,16 +3255,16 @@
         <v>139</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>157</v>
+        <v>155</v>
       </c>
       <c r="E110" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="111" spans="1:5" x14ac:dyDescent="0.3">
@@ -3268,289 +3272,296 @@
         <v>136</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>158</v>
+        <v>156</v>
       </c>
       <c r="E111" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
     </row>
     <row r="112" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
-        <v>243</v>
+        <v>241</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>95</v>
+        <v>93</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>159</v>
+        <v>157</v>
       </c>
       <c r="E112" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="113" spans="1:5" x14ac:dyDescent="0.3">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="4">
         <v>130</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>160</v>
+        <v>158</v>
       </c>
       <c r="E113" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="114" spans="1:5" x14ac:dyDescent="0.3">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>56</v>
+        <v>55</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D114" s="3" t="s">
+        <v>164</v>
+      </c>
+      <c r="E114" t="s">
+        <v>277</v>
+      </c>
+    </row>
+    <row r="115" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A115" s="4" t="s">
+        <v>243</v>
+      </c>
+      <c r="B115" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C115" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D115" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E115" t="s">
+        <v>277</v>
+      </c>
+      <c r="F115" s="5"/>
+    </row>
+    <row r="116" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A116" s="4" t="s">
+        <v>246</v>
+      </c>
+      <c r="B116" s="1" t="s">
+        <v>308</v>
+      </c>
+      <c r="C116" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D116" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E114" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="115" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A115" s="4" t="s">
+      <c r="E116" t="s">
+        <v>277</v>
+      </c>
+      <c r="F116" s="5"/>
+    </row>
+    <row r="117" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A117" s="4" t="s">
+        <v>269</v>
+      </c>
+      <c r="B117" s="1" t="s">
+        <v>306</v>
+      </c>
+      <c r="C117" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D117" s="3" t="s">
+        <v>167</v>
+      </c>
+      <c r="E117" t="s">
+        <v>277</v>
+      </c>
+      <c r="F117" s="5"/>
+    </row>
+    <row r="118" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A118" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B118" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C118" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D118" s="3" t="s">
+        <v>162</v>
+      </c>
+      <c r="E118" t="s">
+        <v>277</v>
+      </c>
+      <c r="F118" s="5"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" s="4" t="s">
         <v>245</v>
       </c>
-      <c r="B115" s="1" t="s">
-        <v>305</v>
-      </c>
-      <c r="C115" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D115" s="3" t="s">
-        <v>167</v>
-      </c>
-      <c r="E115" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="116" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A116" s="4" t="s">
-        <v>248</v>
-      </c>
-      <c r="B116" s="1" t="s">
-        <v>310</v>
-      </c>
-      <c r="C116" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D116" s="3" t="s">
+      <c r="B119" s="1" t="s">
+        <v>309</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D119" s="3" t="s">
         <v>168</v>
       </c>
-      <c r="E116" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="117" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A117" s="4" t="s">
-        <v>247</v>
-      </c>
-      <c r="B117" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="C117" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D117" s="3" t="s">
+      <c r="F119" s="5"/>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="4" t="s">
+        <v>228</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D120" s="3" t="s">
+        <v>163</v>
+      </c>
+      <c r="F120" s="5"/>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" s="4" t="s">
+        <v>244</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>302</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D121" s="3" t="s">
         <v>169</v>
       </c>
-      <c r="E117" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="118" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A118" s="4" t="s">
-        <v>246</v>
-      </c>
-      <c r="B118" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="C118" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D118" s="3" t="s">
-        <v>164</v>
-      </c>
-      <c r="E118" t="s">
-        <v>279</v>
-      </c>
-    </row>
-    <row r="119" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A119" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>311</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>170</v>
-      </c>
-    </row>
-    <row r="120" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A120" s="4" t="s">
-        <v>250</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>306</v>
-      </c>
-      <c r="C120" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D120" s="3" t="s">
-        <v>165</v>
-      </c>
-    </row>
-    <row r="121" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A121" s="4">
-        <v>103</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>304</v>
-      </c>
-      <c r="C121" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D121" s="3" t="s">
-        <v>171</v>
-      </c>
-    </row>
-    <row r="122" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="F121" s="5"/>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="4">
         <v>119</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>309</v>
+        <v>307</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>172</v>
-      </c>
-    </row>
-    <row r="123" spans="1:5" x14ac:dyDescent="0.3">
+        <v>170</v>
+      </c>
+    </row>
+    <row r="123" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A123" s="4">
         <v>148</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>84</v>
+        <v>312</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D123" s="3" t="s">
+        <v>171</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" s="4" t="s">
+        <v>310</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>311</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D124" s="3" t="s">
+        <v>172</v>
+      </c>
+    </row>
+    <row r="125" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A125" s="4" t="s">
+        <v>249</v>
+      </c>
+      <c r="B125" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C125" s="3" t="s">
+        <v>143</v>
+      </c>
+      <c r="D125" s="3" t="s">
         <v>173</v>
       </c>
     </row>
-    <row r="124" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A124" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>174</v>
-      </c>
-    </row>
-    <row r="125" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A125" s="4" t="s">
+    <row r="126" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A126" s="4" t="s">
         <v>251</v>
-      </c>
-      <c r="B125" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C125" s="3" t="s">
-        <v>145</v>
-      </c>
-      <c r="D125" s="3" t="s">
-        <v>175</v>
-      </c>
-    </row>
-    <row r="126" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A126" s="4" t="s">
-        <v>253</v>
       </c>
       <c r="B126" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>176</v>
-      </c>
-    </row>
-    <row r="127" spans="1:5" x14ac:dyDescent="0.3">
+        <v>174</v>
+      </c>
+    </row>
+    <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="4">
         <v>159</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>96</v>
+        <v>94</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>290</v>
-      </c>
-    </row>
-    <row r="128" spans="1:5" x14ac:dyDescent="0.3">
+        <v>288</v>
+      </c>
+    </row>
+    <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="129" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A129" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B129" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="130" spans="1:4" x14ac:dyDescent="0.3">
@@ -3558,27 +3569,27 @@
         <v>157</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>88</v>
+        <v>86</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="131" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A131" s="4" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B131" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="132" spans="1:4" x14ac:dyDescent="0.3">
@@ -3589,24 +3600,24 @@
         <v>4</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="133" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A133" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="134" spans="1:4" x14ac:dyDescent="0.3">
@@ -3617,24 +3628,24 @@
         <v>8</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="135" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B135" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="136" spans="1:4" x14ac:dyDescent="0.3">
@@ -3642,55 +3653,55 @@
         <v>121</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>50</v>
+        <v>49</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="137" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="138" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="139" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="140" spans="1:4" x14ac:dyDescent="0.3">
@@ -3698,13 +3709,13 @@
         <v>113</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="141" spans="1:4" x14ac:dyDescent="0.3">
@@ -3715,10 +3726,10 @@
         <v>7</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="142" spans="1:4" x14ac:dyDescent="0.3">
@@ -3726,13 +3737,13 @@
         <v>102</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="143" spans="1:4" x14ac:dyDescent="0.3">
@@ -3740,13 +3751,13 @@
         <v>156</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>87</v>
+        <v>85</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="144" spans="1:4" x14ac:dyDescent="0.3">
@@ -3754,13 +3765,13 @@
         <v>133</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="145" spans="1:4" x14ac:dyDescent="0.3">
@@ -3768,13 +3779,13 @@
         <v>118</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>48</v>
+        <v>47</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
@@ -3782,27 +3793,27 @@
         <v>123</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>51</v>
+        <v>50</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>146</v>
+        <v>144</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A147" s="4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B147" s="1" t="s">
         <v>3</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
@@ -3810,13 +3821,13 @@
         <v>145</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>147</v>
+        <v>145</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
@@ -3824,13 +3835,13 @@
         <v>135</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C149" s="3" t="s">
+        <v>145</v>
+      </c>
+      <c r="D149" s="3" t="s">
         <v>147</v>
-      </c>
-      <c r="D149" s="3" t="s">
-        <v>149</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
@@ -3838,13 +3849,13 @@
         <v>125</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>163</v>
+        <v>161</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
@@ -3852,125 +3863,125 @@
         <v>143</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>162</v>
+        <v>160</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>148</v>
+        <v>146</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>61</v>
+        <v>60</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="B158" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A159" s="4" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>62</v>
+        <v>61</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
@@ -3978,83 +3989,83 @@
         <v>120</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>49</v>
+        <v>48</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>149</v>
+        <v>147</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>145</v>
+        <v>143</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
-        <v>271</v>
+        <v>247</v>
       </c>
       <c r="B161" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>55</v>
+        <v>54</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>150</v>
+        <v>148</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.3">
@@ -4062,13 +4073,13 @@
         <v>132</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.3">
@@ -4076,13 +4087,13 @@
         <v>129</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.3">
@@ -4090,13 +4101,13 @@
         <v>127</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>142</v>
+        <v>140</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.3">
@@ -4104,13 +4115,13 @@
         <v>169</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.3">
@@ -4118,13 +4129,13 @@
         <v>122</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>151</v>
+        <v>149</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.3">
@@ -4132,13 +4143,13 @@
         <v>171</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>152</v>
+        <v>150</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>161</v>
+        <v>159</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
grammar, up to 138
</commit_message>
<xml_diff>
--- a/p/content_by_grammar.xlsx
+++ b/p/content_by_grammar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adsv\private\books\language\ingush\Dahkilgov\github\dahkilgov\p\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{E5FE850C-8A8C-4797-8466-4A5432F6279B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1E1EE6-2C6E-4BC3-8CB1-12CA48A869FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2415" windowWidth="38640" windowHeight="21120" xr2:uid="{AC639D1C-64A7-45F6-9CFA-A1A688E9895B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="752" uniqueCount="317">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="320">
   <si>
     <t>Причастие, несамостоятельное, настоящее время</t>
   </si>
@@ -116,9 +116,6 @@
     <t>Местоимение, определительное.</t>
   </si>
   <si>
-    <t>Морфология. Сравнение.</t>
-  </si>
-  <si>
     <t>Глагол, времена, настоящее время.</t>
   </si>
   <si>
@@ -281,9 +278,6 @@
     <t>Существительное, падежи, склонение личных имен.</t>
   </si>
   <si>
-    <t>Деепричастие, прошедшее время, отрицательная форма.</t>
-  </si>
-  <si>
     <t>Причастие, несамостоятельное, будущее время.</t>
   </si>
   <si>
@@ -956,12 +950,6 @@
     <t>Деепричастие, соединительный оборот с союзом “а”.</t>
   </si>
   <si>
-    <t>Деепричастие, описательные обороты.</t>
-  </si>
-  <si>
-    <t>Деепричастие, прошедшее время, окончания -е, -ий, -й.</t>
-  </si>
-  <si>
     <t>Глагол, вспомогательный глагол “да” - есть.</t>
   </si>
   <si>
@@ -989,7 +977,28 @@
     <t>перенести отрицание ближе к концу, после ознакомления с терминами причастие, деепричастие, и т.д.</t>
   </si>
   <si>
-    <t>тема уже раскрыта в Притче 96 про прилагательные</t>
+    <t>перенести в начало ?</t>
+  </si>
+  <si>
+    <t>Причастие, примеры разных форм причастий в разных временах.</t>
+  </si>
+  <si>
+    <t>заменить на модальную форму, Ахриева 184</t>
+  </si>
+  <si>
+    <t>заменить на совпадение формы деепричастия с причастием прошедшего времени</t>
+  </si>
+  <si>
+    <t>Деепричастие, отрицательная форма.</t>
+  </si>
+  <si>
+    <t>Деепричастие, описательные обороты для времени действия.</t>
+  </si>
+  <si>
+    <t>Деепричастие, соединительный оборот, окончания -е, -ий, -й.</t>
+  </si>
+  <si>
+    <t>заменить на примеры, переместить сразу после времен</t>
   </si>
 </sst>
 </file>
@@ -1411,36 +1420,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>169</v>
+        <v>167</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>118</v>
+        <v>116</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>170</v>
+        <v>168</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>107</v>
+        <v>105</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1448,16 +1457,16 @@
         <v>144</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>106</v>
+        <v>104</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1465,50 +1474,50 @@
         <v>105</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>171</v>
+        <v>169</v>
       </c>
       <c r="B5" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C5" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="D5" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E5" s="5" t="s">
         <v>270</v>
-      </c>
-      <c r="C5" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="D5" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E5" s="5" t="s">
-        <v>272</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>172</v>
+        <v>170</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>108</v>
+        <v>106</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
@@ -1516,33 +1525,33 @@
         <v>152</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>109</v>
+        <v>107</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E7" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>173</v>
+        <v>171</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>112</v>
+        <v>110</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E8" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
@@ -1550,84 +1559,84 @@
         <v>166</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>117</v>
+        <v>115</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="E9" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>174</v>
+        <v>172</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>119</v>
+        <v>117</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E10" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>175</v>
+        <v>173</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>120</v>
+        <v>118</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E11" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>176</v>
+        <v>174</v>
       </c>
       <c r="B12" s="1" t="s">
+        <v>127</v>
+      </c>
+      <c r="C12" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D12" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="C12" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D12" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="E12" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>177</v>
+        <v>175</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>125</v>
+        <v>123</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E13" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
@@ -1635,16 +1644,16 @@
         <v>124</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>122</v>
+        <v>120</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E14" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
@@ -1652,16 +1661,16 @@
         <v>116</v>
       </c>
       <c r="B15" s="1" t="s">
-        <v>123</v>
+        <v>121</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="E15" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
@@ -1669,291 +1678,291 @@
         <v>128</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>127</v>
+        <v>125</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="E16" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>178</v>
+        <v>176</v>
       </c>
       <c r="B17" s="1" t="s">
-        <v>121</v>
+        <v>119</v>
       </c>
       <c r="C17" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="D17" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D17" s="3" t="s">
-        <v>133</v>
-      </c>
       <c r="E17" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>179</v>
+        <v>177</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>126</v>
+        <v>124</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="E18" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>180</v>
+        <v>178</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>124</v>
+        <v>122</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="E19" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>181</v>
+        <v>179</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>128</v>
+        <v>126</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="E20" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>182</v>
+        <v>180</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>113</v>
+        <v>111</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
       <c r="E21" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>183</v>
+        <v>181</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>114</v>
+        <v>112</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
       <c r="E22" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>25</v>
+        <v>19</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
+      </c>
+      <c r="E23" t="s">
+        <v>269</v>
       </c>
       <c r="F23" t="s">
-        <v>316</v>
+        <v>311</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4" t="s">
-        <v>185</v>
+      <c r="A24" s="4">
+        <v>165</v>
       </c>
       <c r="B24" s="1" t="s">
-        <v>19</v>
+        <v>101</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>133</v>
+        <v>130</v>
       </c>
       <c r="E24" t="s">
-        <v>271</v>
-      </c>
-      <c r="F24" t="s">
-        <v>315</v>
+        <v>269</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4">
-        <v>165</v>
+        <v>137</v>
       </c>
       <c r="B25" s="1" t="s">
-        <v>103</v>
+        <v>271</v>
       </c>
       <c r="C25" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E25" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>184</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="D26" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="D25" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E25" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4">
-        <v>137</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="E26" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>15</v>
+        <v>272</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>136</v>
+        <v>133</v>
       </c>
       <c r="E27" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="4" t="s">
-        <v>187</v>
+      <c r="A28" s="4">
+        <v>138</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>274</v>
+        <v>72</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>137</v>
+        <v>134</v>
       </c>
       <c r="E28" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4">
-        <v>138</v>
+        <v>117</v>
       </c>
       <c r="B29" s="1" t="s">
-        <v>73</v>
+        <v>273</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>138</v>
+        <v>135</v>
       </c>
       <c r="E29" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4">
-        <v>117</v>
+      <c r="A30" s="4" t="s">
+        <v>186</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>275</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>139</v>
+        <v>136</v>
       </c>
       <c r="E30" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>188</v>
+      <c r="A31" s="4">
+        <v>147</v>
       </c>
       <c r="B31" s="1" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>140</v>
+        <v>137</v>
       </c>
       <c r="E31" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="4">
-        <v>147</v>
+      <c r="A32" s="4" t="s">
+        <v>187</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>276</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>141</v>
+        <v>138</v>
       </c>
       <c r="E32" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
@@ -1961,169 +1970,169 @@
         <v>189</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>278</v>
+        <v>91</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>142</v>
+        <v>151</v>
       </c>
       <c r="E33" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
+        <v>190</v>
+      </c>
+      <c r="B34" s="1" t="s">
+        <v>39</v>
+      </c>
+      <c r="C34" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D34" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E34" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A35" s="4">
+        <v>114</v>
+      </c>
+      <c r="B35" s="1" t="s">
+        <v>44</v>
+      </c>
+      <c r="C35" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D35" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E35" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A36" s="4" t="s">
         <v>191</v>
       </c>
-      <c r="B34" s="1" t="s">
-        <v>93</v>
-      </c>
-      <c r="C34" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D34" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E34" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="4" t="s">
-        <v>192</v>
-      </c>
-      <c r="B35" s="1" t="s">
-        <v>40</v>
-      </c>
-      <c r="C35" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D35" s="3" t="s">
+      <c r="B36" s="1" t="s">
+        <v>94</v>
+      </c>
+      <c r="C36" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D36" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E35" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="36" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A36" s="4">
-        <v>114</v>
-      </c>
-      <c r="B36" s="1" t="s">
-        <v>45</v>
-      </c>
-      <c r="C36" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D36" s="3" t="s">
-        <v>131</v>
-      </c>
       <c r="E36" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>96</v>
+        <v>11</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E37" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>11</v>
+        <v>277</v>
       </c>
       <c r="C38" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D38" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E38" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A39" s="4">
+        <v>134</v>
+      </c>
+      <c r="B39" s="1" t="s">
+        <v>97</v>
+      </c>
+      <c r="C39" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="D38" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E38" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="39" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A39" s="4" t="s">
-        <v>195</v>
-      </c>
-      <c r="B39" s="1" t="s">
-        <v>279</v>
-      </c>
-      <c r="C39" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>134</v>
-      </c>
       <c r="E39" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A40" s="4">
+        <v>106</v>
+      </c>
+      <c r="B40" s="1" t="s">
+        <v>41</v>
+      </c>
+      <c r="C40" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D40" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="B40" s="1" t="s">
-        <v>99</v>
-      </c>
-      <c r="C40" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D40" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="E40" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A41" s="4">
-        <v>106</v>
+      <c r="A41" s="4" t="s">
+        <v>188</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>42</v>
+        <v>278</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E41" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>190</v>
+        <v>194</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>280</v>
+        <v>92</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="E42" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
@@ -2131,1369 +2140,1369 @@
         <v>196</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>94</v>
+        <v>34</v>
       </c>
       <c r="C43" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D43" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="E43" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>35</v>
+        <v>32</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
       <c r="E44" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>33</v>
+        <v>20</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="E45" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>20</v>
+        <v>61</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="E46" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>62</v>
+        <v>33</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="E47" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="48" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>34</v>
+        <v>95</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D48" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E48" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A49" s="4">
+        <v>141</v>
+      </c>
+      <c r="B49" s="1" t="s">
+        <v>96</v>
+      </c>
+      <c r="C49" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D49" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E48" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="49" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A49" s="4" t="s">
-        <v>203</v>
-      </c>
-      <c r="B49" s="1" t="s">
-        <v>97</v>
-      </c>
-      <c r="C49" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D49" s="3" t="s">
-        <v>144</v>
-      </c>
       <c r="E49" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>98</v>
+        <v>81</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
       <c r="E50" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>83</v>
+        <v>78</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
       <c r="E51" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>79</v>
+        <v>82</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
       <c r="E52" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A53" s="4">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>84</v>
+        <v>93</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D53" s="3" t="s">
+        <v>147</v>
+      </c>
+      <c r="E53" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A54" s="4" t="s">
+        <v>195</v>
+      </c>
+      <c r="B54" s="1" t="s">
+        <v>62</v>
+      </c>
+      <c r="C54" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="D54" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E53" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="54" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A54" s="4">
-        <v>154</v>
-      </c>
-      <c r="B54" s="1" t="s">
-        <v>95</v>
-      </c>
-      <c r="C54" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D54" s="3" t="s">
-        <v>149</v>
-      </c>
       <c r="E54" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>197</v>
+        <v>202</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>63</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E55" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>64</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="E56" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>65</v>
+        <v>279</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E57" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>281</v>
+        <v>66</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E58" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A59" s="4" t="s">
-        <v>207</v>
+      <c r="A59" s="4">
+        <v>100</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>67</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E59" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A60" s="4">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>68</v>
+        <v>280</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E60" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A61" s="4">
-        <v>101</v>
+      <c r="A61" s="4" t="s">
+        <v>240</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>282</v>
+        <v>281</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="E61" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>242</v>
+        <v>283</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>283</v>
+        <v>284</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E62" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>285</v>
+        <v>206</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>286</v>
+        <v>17</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>162</v>
+        <v>151</v>
       </c>
       <c r="E63" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B64" s="1" t="s">
-        <v>17</v>
+        <v>37</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="E64" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>38</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
       <c r="D65" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E65" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A66" s="4">
+        <v>142</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>71</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D66" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E65" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="4" t="s">
+      <c r="E66" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A67" s="4" t="s">
+        <v>209</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>285</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E67" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A68" s="4">
+        <v>126</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>69</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E68" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A69" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B66" s="1" t="s">
-        <v>39</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E66" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="4">
-        <v>142</v>
-      </c>
-      <c r="B67" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D67" s="3" t="s">
+      <c r="B69" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C69" s="3" t="s">
         <v>132</v>
       </c>
-      <c r="E67" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D68" s="3" t="s">
+      <c r="D69" s="3" t="s">
         <v>133</v>
       </c>
-      <c r="E68" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="4">
-        <v>126</v>
-      </c>
-      <c r="B69" s="1" t="s">
-        <v>70</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>134</v>
-      </c>
       <c r="E69" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
+        <v>211</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>286</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="E70" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A71" s="4">
+        <v>151</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>98</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E71" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A72" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="B70" s="1" t="s">
-        <v>54</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E70" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="4" t="s">
+      <c r="B72" s="1" t="s">
+        <v>58</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E72" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A73" s="4">
+        <v>149</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>6</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E73" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A74" s="4" t="s">
         <v>213</v>
       </c>
-      <c r="B71" s="1" t="s">
+      <c r="B74" s="1" t="s">
+        <v>12</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="E74" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A75" s="4">
+        <v>107</v>
+      </c>
+      <c r="B75" s="1" t="s">
         <v>288</v>
       </c>
-      <c r="C71" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E71" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="4">
-        <v>151</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>100</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E72" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>59</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E73" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="4">
-        <v>149</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E74" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>12</v>
-      </c>
       <c r="C75" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="E75" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="4">
-        <v>107</v>
+        <v>164</v>
       </c>
       <c r="B76" s="1" t="s">
+        <v>289</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E76" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>214</v>
+      </c>
+      <c r="B77" s="1" t="s">
         <v>290</v>
       </c>
-      <c r="C76" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D76" s="3" t="s">
+      <c r="C77" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D77" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E76" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="4">
-        <v>164</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>291</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D77" s="3" t="s">
+      <c r="E77" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A78" s="4">
+        <v>111</v>
+      </c>
+      <c r="B78" s="1" t="s">
+        <v>287</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="D78" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E77" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="4" t="s">
-        <v>216</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>292</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>132</v>
-      </c>
       <c r="E78" t="s">
-        <v>271</v>
+        <v>269</v>
+      </c>
+      <c r="F78" t="s">
+        <v>306</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="4">
-        <v>111</v>
+      <c r="A79" s="4" t="s">
+        <v>215</v>
       </c>
       <c r="B79" s="1" t="s">
-        <v>289</v>
+        <v>9</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>133</v>
+        <v>151</v>
       </c>
       <c r="E79" t="s">
-        <v>271</v>
-      </c>
-      <c r="F79" t="s">
-        <v>310</v>
+        <v>269</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>9</v>
+        <v>36</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="E80" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>37</v>
+        <v>21</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E81" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>21</v>
+        <v>55</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
       <c r="E82" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>56</v>
+        <v>23</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
       <c r="E83" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>221</v>
+        <v>282</v>
       </c>
       <c r="B84" s="1" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
       <c r="E84" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>284</v>
+        <v>221</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>24</v>
+        <v>28</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D85" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E85" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A86" s="4">
+        <v>158</v>
+      </c>
+      <c r="B86" s="1" t="s">
+        <v>80</v>
+      </c>
+      <c r="C86" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E85" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="86" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A86" s="4" t="s">
-        <v>223</v>
-      </c>
-      <c r="B86" s="1" t="s">
-        <v>29</v>
-      </c>
-      <c r="C86" s="3" t="s">
-        <v>136</v>
-      </c>
       <c r="D86" s="3" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="E86" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>82</v>
+        <v>74</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="E87" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A88" s="4">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>75</v>
+        <v>5</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>137</v>
+        <v>151</v>
       </c>
       <c r="E88" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A89" s="4">
-        <v>112</v>
+      <c r="A89" s="4" t="s">
+        <v>222</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>5</v>
+        <v>35</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="E89" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>36</v>
+        <v>84</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
       <c r="E90" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
+        <v>224</v>
+      </c>
+      <c r="B91" s="1" t="s">
+        <v>25</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E91" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A92" s="4">
+        <v>108</v>
+      </c>
+      <c r="B92" s="1" t="s">
+        <v>88</v>
+      </c>
+      <c r="C92" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D92" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E92" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A93" s="4" t="s">
         <v>225</v>
       </c>
-      <c r="B91" s="1" t="s">
-        <v>86</v>
-      </c>
-      <c r="C91" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E91" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" s="4" t="s">
+      <c r="B93" s="1" t="s">
+        <v>29</v>
+      </c>
+      <c r="C93" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D93" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E93" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A94" s="4">
+        <v>110</v>
+      </c>
+      <c r="B94" s="1" t="s">
+        <v>42</v>
+      </c>
+      <c r="C94" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D94" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E94" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A95" s="4" t="s">
         <v>226</v>
       </c>
-      <c r="B92" s="1" t="s">
-        <v>26</v>
-      </c>
-      <c r="C92" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D92" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E92" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="4">
-        <v>108</v>
-      </c>
-      <c r="B93" s="1" t="s">
-        <v>90</v>
-      </c>
-      <c r="C93" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D93" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E93" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="94" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A94" s="4" t="s">
-        <v>227</v>
-      </c>
-      <c r="B94" s="1" t="s">
-        <v>30</v>
-      </c>
-      <c r="C94" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D94" s="3" t="s">
+      <c r="B95" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C95" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D95" s="3" t="s">
         <v>134</v>
       </c>
-      <c r="E94" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="95" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A95" s="4">
-        <v>110</v>
-      </c>
-      <c r="B95" s="1" t="s">
-        <v>43</v>
-      </c>
-      <c r="C95" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D95" s="3" t="s">
-        <v>135</v>
-      </c>
       <c r="E95" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
+        <v>227</v>
+      </c>
+      <c r="B96" s="1" t="s">
+        <v>26</v>
+      </c>
+      <c r="C96" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D96" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E96" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="97" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A97" s="4" t="s">
         <v>228</v>
       </c>
-      <c r="B96" s="1" t="s">
+      <c r="B97" s="1" t="s">
+        <v>40</v>
+      </c>
+      <c r="C97" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D97" s="3" t="s">
+        <v>136</v>
+      </c>
+      <c r="E97" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="98" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A98" s="4">
+        <v>168</v>
+      </c>
+      <c r="B98" s="1" t="s">
+        <v>83</v>
+      </c>
+      <c r="C98" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D98" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="E98" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="99" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A99" s="4" t="s">
+        <v>229</v>
+      </c>
+      <c r="B99" s="1" t="s">
         <v>49</v>
       </c>
-      <c r="C96" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D96" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E96" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="97" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A97" s="4" t="s">
-        <v>229</v>
-      </c>
-      <c r="B97" s="1" t="s">
-        <v>27</v>
-      </c>
-      <c r="C97" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D97" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E97" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="98" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A98" s="4" t="s">
+      <c r="C99" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D99" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="E99" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="100" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A100" s="4">
+        <v>104</v>
+      </c>
+      <c r="B100" s="1" t="s">
+        <v>89</v>
+      </c>
+      <c r="C100" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D100" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="E100" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="101" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A101" s="4" t="s">
+        <v>231</v>
+      </c>
+      <c r="B101" s="1" t="s">
+        <v>47</v>
+      </c>
+      <c r="C101" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D101" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="E101" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="102" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A102" s="4" t="s">
         <v>230</v>
       </c>
-      <c r="B98" s="1" t="s">
-        <v>41</v>
-      </c>
-      <c r="C98" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D98" s="3" t="s">
-        <v>138</v>
-      </c>
-      <c r="E98" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="99" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A99" s="4">
-        <v>168</v>
-      </c>
-      <c r="B99" s="1" t="s">
-        <v>85</v>
-      </c>
-      <c r="C99" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D99" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="E99" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="100" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A100" s="4" t="s">
-        <v>231</v>
-      </c>
-      <c r="B100" s="1" t="s">
-        <v>50</v>
-      </c>
-      <c r="C100" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D100" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="E100" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="101" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A101" s="4">
-        <v>104</v>
-      </c>
-      <c r="B101" s="1" t="s">
-        <v>91</v>
-      </c>
-      <c r="C101" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D101" s="3" t="s">
+      <c r="B102" s="1" t="s">
+        <v>90</v>
+      </c>
+      <c r="C102" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="E101" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="102" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A102" s="4" t="s">
-        <v>233</v>
-      </c>
-      <c r="B102" s="1" t="s">
-        <v>48</v>
-      </c>
-      <c r="C102" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D102" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="E102" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="103" spans="1:5" x14ac:dyDescent="0.3">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
         <v>232</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>92</v>
+        <v>54</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D103" s="3" t="s">
+        <v>142</v>
+      </c>
+      <c r="E103" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="104" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A104" s="4">
+        <v>153</v>
+      </c>
+      <c r="B104" s="1" t="s">
+        <v>77</v>
+      </c>
+      <c r="C104" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D104" s="3" t="s">
         <v>143</v>
       </c>
-      <c r="E103" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="104" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A104" s="4" t="s">
-        <v>234</v>
-      </c>
-      <c r="B104" s="1" t="s">
-        <v>55</v>
-      </c>
-      <c r="C104" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D104" s="3" t="s">
+      <c r="E104" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="105" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A105" s="4">
+        <v>146</v>
+      </c>
+      <c r="B105" s="1" t="s">
+        <v>76</v>
+      </c>
+      <c r="C105" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D105" s="3" t="s">
         <v>144</v>
       </c>
-      <c r="E104" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="105" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A105" s="4">
-        <v>153</v>
-      </c>
-      <c r="B105" s="1" t="s">
-        <v>78</v>
-      </c>
-      <c r="C105" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D105" s="3" t="s">
+      <c r="E105" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="106" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A106" s="4">
+        <v>115</v>
+      </c>
+      <c r="B106" s="1" t="s">
+        <v>87</v>
+      </c>
+      <c r="C106" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D106" s="3" t="s">
         <v>145</v>
       </c>
-      <c r="E105" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="106" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A106" s="4">
+      <c r="E106" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="107" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A107" s="4">
+        <v>139</v>
+      </c>
+      <c r="B107" s="1" t="s">
+        <v>73</v>
+      </c>
+      <c r="C107" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D107" s="3" t="s">
         <v>146</v>
       </c>
-      <c r="B106" s="1" t="s">
-        <v>77</v>
-      </c>
-      <c r="C106" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D106" s="3" t="s">
-        <v>146</v>
-      </c>
-      <c r="E106" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="107" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A107" s="4">
-        <v>115</v>
-      </c>
-      <c r="B107" s="1" t="s">
-        <v>89</v>
-      </c>
-      <c r="C107" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D107" s="3" t="s">
+      <c r="E107" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="108" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A108" s="4">
+        <v>136</v>
+      </c>
+      <c r="B108" s="1" t="s">
+        <v>291</v>
+      </c>
+      <c r="C108" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D108" s="3" t="s">
         <v>147</v>
       </c>
-      <c r="E107" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="108" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A108" s="4">
-        <v>139</v>
-      </c>
-      <c r="B108" s="1" t="s">
-        <v>74</v>
-      </c>
-      <c r="C108" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D108" s="3" t="s">
+      <c r="E108" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="109" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A109" s="4" t="s">
+        <v>233</v>
+      </c>
+      <c r="B109" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C109" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D109" s="3" t="s">
         <v>148</v>
       </c>
-      <c r="E108" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="109" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A109" s="4">
-        <v>136</v>
-      </c>
-      <c r="B109" s="1" t="s">
+      <c r="E109" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="110" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A110" s="4">
+        <v>130</v>
+      </c>
+      <c r="B110" s="1" t="s">
+        <v>70</v>
+      </c>
+      <c r="C110" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D110" s="3" t="s">
+        <v>149</v>
+      </c>
+      <c r="E110" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="111" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A111" s="4" t="s">
+        <v>242</v>
+      </c>
+      <c r="B111" s="1" t="s">
+        <v>51</v>
+      </c>
+      <c r="C111" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D111" s="3" t="s">
+        <v>150</v>
+      </c>
+      <c r="E111" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="112" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A112" s="4" t="s">
+        <v>235</v>
+      </c>
+      <c r="B112" s="1" t="s">
         <v>293</v>
       </c>
-      <c r="C109" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D109" s="3" t="s">
-        <v>149</v>
-      </c>
-      <c r="E109" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="110" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A110" s="4" t="s">
-        <v>235</v>
-      </c>
-      <c r="B110" s="1" t="s">
-        <v>87</v>
-      </c>
-      <c r="C110" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D110" s="3" t="s">
-        <v>150</v>
-      </c>
-      <c r="E110" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="111" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A111" s="4">
-        <v>130</v>
-      </c>
-      <c r="B111" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C111" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D111" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E111" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="112" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A112" s="4" t="s">
-        <v>244</v>
-      </c>
-      <c r="B112" s="1" t="s">
-        <v>52</v>
-      </c>
       <c r="C112" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>152</v>
+        <v>156</v>
       </c>
       <c r="E112" t="s">
-        <v>271</v>
-      </c>
+        <v>269</v>
+      </c>
+      <c r="F112" s="5"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
-        <v>237</v>
+        <v>238</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>295</v>
+        <v>297</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="E113" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F113" s="5"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>240</v>
+        <v>261</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="E114" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F114" s="5"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
-        <v>263</v>
+        <v>234</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="E115" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F115" s="5"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
-        <v>236</v>
+        <v>237</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>297</v>
+        <v>298</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>161</v>
+        <v>154</v>
       </c>
       <c r="E116" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F116" s="5"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
-        <v>239</v>
+        <v>220</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>300</v>
+        <v>294</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>156</v>
+        <v>160</v>
       </c>
       <c r="E117" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="F117" s="5"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
-        <v>222</v>
+        <v>236</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>296</v>
+        <v>292</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D118" s="3" t="s">
+        <v>155</v>
+      </c>
+      <c r="E118" t="s">
+        <v>269</v>
+      </c>
+      <c r="F118" s="5"/>
+    </row>
+    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A119" s="4">
+        <v>131</v>
+      </c>
+      <c r="B119" s="1" t="s">
+        <v>305</v>
+      </c>
+      <c r="C119" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D119" s="3" t="s">
+        <v>161</v>
+      </c>
+      <c r="E119" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A120" s="4" t="s">
+        <v>299</v>
+      </c>
+      <c r="B120" s="1" t="s">
+        <v>303</v>
+      </c>
+      <c r="C120" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D120" s="3" t="s">
         <v>162</v>
       </c>
-      <c r="E118" t="s">
-        <v>271</v>
-      </c>
-      <c r="F118" s="5"/>
-    </row>
-    <row r="119" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A119" s="4" t="s">
-        <v>238</v>
-      </c>
-      <c r="B119" s="1" t="s">
-        <v>294</v>
-      </c>
-      <c r="C119" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D119" s="3" t="s">
-        <v>157</v>
-      </c>
-      <c r="E119" t="s">
-        <v>271</v>
-      </c>
-      <c r="F119" s="5"/>
-    </row>
-    <row r="120" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A120" s="4">
-        <v>131</v>
-      </c>
-      <c r="B120" s="1" t="s">
-        <v>309</v>
-      </c>
-      <c r="C120" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D120" s="3" t="s">
+      <c r="E120" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A121" s="4">
+        <v>148</v>
+      </c>
+      <c r="B121" s="1" t="s">
+        <v>304</v>
+      </c>
+      <c r="C121" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D121" s="3" t="s">
         <v>163</v>
       </c>
-      <c r="E120" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="121" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A121" s="4" t="s">
-        <v>301</v>
-      </c>
-      <c r="B121" s="1" t="s">
-        <v>307</v>
-      </c>
-      <c r="C121" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D121" s="3" t="s">
+      <c r="E121" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A122" s="4" t="s">
+        <v>241</v>
+      </c>
+      <c r="B122" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C122" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D122" s="3" t="s">
         <v>164</v>
       </c>
-      <c r="E121" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="122" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A122" s="4">
-        <v>148</v>
-      </c>
-      <c r="B122" s="1" t="s">
-        <v>308</v>
-      </c>
-      <c r="C122" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D122" s="3" t="s">
-        <v>165</v>
-      </c>
       <c r="E122" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
@@ -3501,208 +3510,226 @@
         <v>243</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>66</v>
+        <v>31</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>137</v>
+        <v>135</v>
       </c>
       <c r="D123" s="3" t="s">
+        <v>165</v>
+      </c>
+      <c r="E123" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A124" s="4">
+        <v>159</v>
+      </c>
+      <c r="B124" s="1" t="s">
+        <v>86</v>
+      </c>
+      <c r="C124" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="D124" s="3" t="s">
         <v>166</v>
       </c>
-      <c r="E123" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="124" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A124" s="4" t="s">
-        <v>245</v>
-      </c>
-      <c r="B124" s="1" t="s">
-        <v>32</v>
-      </c>
-      <c r="C124" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="D124" s="3" t="s">
-        <v>167</v>
-      </c>
       <c r="E124" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A125" s="4">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>88</v>
+        <v>153</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>168</v>
+        <v>151</v>
       </c>
       <c r="E125" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A126" s="4">
-        <v>125</v>
+        <v>143</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>155</v>
+        <v>152</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>138</v>
+        <v>136</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>153</v>
+        <v>128</v>
       </c>
       <c r="E126" t="s">
-        <v>271</v>
+        <v>269</v>
+      </c>
+      <c r="F126" t="s">
+        <v>307</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A127" s="4">
-        <v>143</v>
+      <c r="A127" s="4" t="s">
+        <v>244</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>154</v>
+        <v>52</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>130</v>
+        <v>151</v>
       </c>
       <c r="E127" t="s">
-        <v>271</v>
-      </c>
-      <c r="F127" t="s">
-        <v>311</v>
+        <v>269</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A128" s="4" t="s">
+        <v>245</v>
+      </c>
+      <c r="B128" s="1" t="s">
+        <v>0</v>
+      </c>
+      <c r="C128" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D128" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E128" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A129" s="4">
+        <v>157</v>
+      </c>
+      <c r="B129" s="1" t="s">
+        <v>79</v>
+      </c>
+      <c r="C129" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D129" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E129" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A130" s="4" t="s">
         <v>246</v>
       </c>
-      <c r="B128" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C128" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D128" s="3" t="s">
-        <v>153</v>
-      </c>
-      <c r="E128" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="4" t="s">
+      <c r="B130" s="1" t="s">
+        <v>1</v>
+      </c>
+      <c r="C130" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D130" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E130" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A131" s="4">
+        <v>109</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>4</v>
+      </c>
+      <c r="C131" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D131" s="3" t="s">
+        <v>131</v>
+      </c>
+      <c r="E131" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A132" s="4" t="s">
         <v>247</v>
       </c>
-      <c r="B129" s="1" t="s">
-        <v>0</v>
-      </c>
-      <c r="C129" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D129" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E129" t="s">
-        <v>271</v>
-      </c>
-    </row>
-    <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="4">
-        <v>157</v>
-      </c>
-      <c r="B130" s="1" t="s">
-        <v>81</v>
-      </c>
-      <c r="C130" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D130" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="4" t="s">
+      <c r="B132" s="1" t="s">
+        <v>60</v>
+      </c>
+      <c r="C132" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D132" s="3" t="s">
+        <v>132</v>
+      </c>
+      <c r="E132" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A133" s="4">
+        <v>161</v>
+      </c>
+      <c r="B133" s="1" t="s">
+        <v>8</v>
+      </c>
+      <c r="C133" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D133" s="3" t="s">
+        <v>133</v>
+      </c>
+      <c r="E133" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A134" s="4" t="s">
         <v>248</v>
       </c>
-      <c r="B131" s="1" t="s">
-        <v>1</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D131" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="4">
-        <v>109</v>
-      </c>
-      <c r="B132" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C132" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D132" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="4" t="s">
-        <v>249</v>
-      </c>
-      <c r="B133" s="1" t="s">
-        <v>61</v>
-      </c>
-      <c r="C133" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D133" s="3" t="s">
+      <c r="B134" s="1" t="s">
+        <v>313</v>
+      </c>
+      <c r="C134" s="3" t="s">
+        <v>137</v>
+      </c>
+      <c r="D134" s="3" t="s">
         <v>134</v>
       </c>
-    </row>
-    <row r="134" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A134" s="4">
-        <v>161</v>
-      </c>
-      <c r="B134" s="1" t="s">
-        <v>8</v>
-      </c>
-      <c r="C134" s="3" t="s">
-        <v>139</v>
-      </c>
-      <c r="D134" s="3" t="s">
-        <v>135</v>
+      <c r="E134" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A135" s="4" t="s">
-        <v>250</v>
+        <v>182</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>313</v>
+        <v>309</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>136</v>
+        <v>135</v>
+      </c>
+      <c r="E135" t="s">
+        <v>269</v>
       </c>
       <c r="F135" t="s">
-        <v>314</v>
+        <v>310</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
@@ -3710,55 +3737,67 @@
         <v>121</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>312</v>
+        <v>308</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
+      </c>
+      <c r="E136" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
-        <v>251</v>
+        <v>249</v>
       </c>
       <c r="B137" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
+      </c>
+      <c r="E137" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A138" s="4" t="s">
-        <v>252</v>
+        <v>250</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>60</v>
+        <v>59</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
+      </c>
+      <c r="E138" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A139" s="4" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="B139" s="1" t="s">
         <v>2</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
+      </c>
+      <c r="F139" t="s">
+        <v>315</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
@@ -3766,13 +3805,16 @@
         <v>113</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>44</v>
+        <v>43</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
+      </c>
+      <c r="E140" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
@@ -3783,10 +3825,13 @@
         <v>7</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
+      </c>
+      <c r="F141" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
@@ -3794,13 +3839,16 @@
         <v>102</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
+      </c>
+      <c r="E142" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
@@ -3808,86 +3856,101 @@
         <v>156</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>80</v>
+        <v>316</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
+      </c>
+      <c r="E143" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A144" s="4">
-        <v>133</v>
+        <v>123</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>306</v>
+        <v>46</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D144" s="3" t="s">
+        <v>134</v>
+      </c>
+      <c r="F144" t="s">
+        <v>319</v>
+      </c>
+    </row>
+    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A145" s="4" t="s">
+        <v>252</v>
+      </c>
+      <c r="B145" s="1" t="s">
+        <v>3</v>
+      </c>
+      <c r="C145" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D145" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E145" t="s">
+        <v>269</v>
+      </c>
+    </row>
+    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A146" s="4">
+        <v>145</v>
+      </c>
+      <c r="B146" s="1" t="s">
+        <v>75</v>
+      </c>
+      <c r="C146" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D146" s="3" t="s">
         <v>136</v>
       </c>
-    </row>
-    <row r="145" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A145" s="4">
-        <v>123</v>
-      </c>
-      <c r="B145" s="1" t="s">
-        <v>47</v>
-      </c>
-      <c r="C145" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D145" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="146" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A146" s="4" t="s">
-        <v>254</v>
-      </c>
-      <c r="B146" s="1" t="s">
-        <v>3</v>
-      </c>
-      <c r="C146" s="3" t="s">
-        <v>140</v>
-      </c>
-      <c r="D146" s="3" t="s">
-        <v>138</v>
+      <c r="E146" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A147" s="4">
-        <v>145</v>
+        <v>135</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>76</v>
+        <v>317</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>139</v>
+        <v>137</v>
+      </c>
+      <c r="E147" t="s">
+        <v>269</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A148" s="4">
-        <v>135</v>
+        <v>133</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>305</v>
+        <v>318</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="E148" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
@@ -3895,16 +3958,16 @@
         <v>118</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>304</v>
+        <v>302</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="E149" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
@@ -3912,16 +3975,16 @@
         <v>160</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>302</v>
+        <v>300</v>
       </c>
       <c r="C150" s="3" t="s">
+        <v>138</v>
+      </c>
+      <c r="D150" s="3" t="s">
         <v>140</v>
       </c>
-      <c r="D150" s="3" t="s">
-        <v>142</v>
-      </c>
       <c r="E150" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -3929,128 +3992,128 @@
         <v>119</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>303</v>
+        <v>301</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>140</v>
+        <v>138</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="E151" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="B152" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="B153" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>130</v>
+        <v>128</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="B154" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>131</v>
+        <v>129</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="B155" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>132</v>
+        <v>130</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="B156" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>133</v>
+        <v>131</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>57</v>
+        <v>56</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>134</v>
+        <v>132</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>28</v>
+        <v>27</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>135</v>
+        <v>133</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="4" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>58</v>
+        <v>57</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>141</v>
+        <v>139</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>136</v>
+        <v>134</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
@@ -4058,167 +4121,179 @@
         <v>120</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>46</v>
+        <v>45</v>
       </c>
       <c r="C160" s="3" t="s">
+        <v>139</v>
+      </c>
+      <c r="D160" s="3" t="s">
+        <v>135</v>
+      </c>
+    </row>
+    <row r="161" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A161" s="4" t="s">
+        <v>239</v>
+      </c>
+      <c r="B161" s="1" t="s">
+        <v>30</v>
+      </c>
+      <c r="C161" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D161" s="3" t="s">
+        <v>151</v>
+      </c>
+    </row>
+    <row r="162" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A162" s="4" t="s">
+        <v>262</v>
+      </c>
+      <c r="B162" s="1" t="s">
+        <v>50</v>
+      </c>
+      <c r="C162" s="3" t="s">
+        <v>140</v>
+      </c>
+      <c r="D162" s="3" t="s">
+        <v>128</v>
+      </c>
+    </row>
+    <row r="163" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A163" s="4" t="s">
+        <v>263</v>
+      </c>
+      <c r="B163" s="1" t="s">
+        <v>114</v>
+      </c>
+      <c r="C163" s="3" t="s">
         <v>141</v>
       </c>
-      <c r="D160" s="3" t="s">
-        <v>137</v>
-      </c>
-    </row>
-    <row r="161" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A161" s="4" t="s">
-        <v>241</v>
-      </c>
-      <c r="B161" s="1" t="s">
-        <v>31</v>
-      </c>
-      <c r="C161" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D161" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="162" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A162" s="4" t="s">
+      <c r="D163" s="3" t="s">
+        <v>151</v>
+      </c>
+      <c r="F163" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="164" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A164" s="4" t="s">
         <v>264</v>
       </c>
-      <c r="B162" s="1" t="s">
-        <v>51</v>
-      </c>
-      <c r="C162" s="3" t="s">
-        <v>142</v>
-      </c>
-      <c r="D162" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="163" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A163" s="4" t="s">
+      <c r="B164" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C164" s="3" t="s">
+        <v>141</v>
+      </c>
+      <c r="D164" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="F164" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="165" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A165" s="4" t="s">
         <v>265</v>
       </c>
-      <c r="B163" s="1" t="s">
-        <v>116</v>
-      </c>
-      <c r="C163" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D163" s="3" t="s">
-        <v>153</v>
-      </c>
-    </row>
-    <row r="164" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A164" s="4" t="s">
-        <v>266</v>
-      </c>
-      <c r="B164" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C164" s="3" t="s">
-        <v>143</v>
-      </c>
-      <c r="D164" s="3" t="s">
-        <v>130</v>
-      </c>
-    </row>
-    <row r="165" spans="1:4" x14ac:dyDescent="0.3">
-      <c r="A165" s="4" t="s">
-        <v>267</v>
-      </c>
       <c r="B165" s="1" t="s">
-        <v>110</v>
+        <v>108</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>131</v>
-      </c>
-    </row>
-    <row r="166" spans="1:4" x14ac:dyDescent="0.3">
+        <v>129</v>
+      </c>
+      <c r="F165" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="166" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A166" s="4">
         <v>132</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>105</v>
+        <v>103</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>132</v>
-      </c>
-    </row>
-    <row r="167" spans="1:4" x14ac:dyDescent="0.3">
+        <v>130</v>
+      </c>
+      <c r="F166" t="s">
+        <v>312</v>
+      </c>
+    </row>
+    <row r="167" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A167" s="4">
         <v>129</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>102</v>
+        <v>100</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>133</v>
-      </c>
-    </row>
-    <row r="168" spans="1:4" x14ac:dyDescent="0.3">
+        <v>131</v>
+      </c>
+    </row>
+    <row r="168" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A168" s="4">
         <v>127</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>101</v>
+        <v>99</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>134</v>
-      </c>
-    </row>
-    <row r="169" spans="1:4" x14ac:dyDescent="0.3">
+        <v>132</v>
+      </c>
+    </row>
+    <row r="169" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A169" s="4">
         <v>169</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>115</v>
+        <v>113</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>135</v>
-      </c>
-    </row>
-    <row r="170" spans="1:4" x14ac:dyDescent="0.3">
+        <v>133</v>
+      </c>
+    </row>
+    <row r="170" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A170" s="4">
         <v>122</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>104</v>
+        <v>102</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>143</v>
+        <v>141</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>136</v>
-      </c>
-    </row>
-    <row r="171" spans="1:4" x14ac:dyDescent="0.3">
+        <v>134</v>
+      </c>
+    </row>
+    <row r="171" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A171" s="4">
         <v>171</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>144</v>
+        <v>142</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>153</v>
+        <v>151</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
grammar, up to 162
</commit_message>
<xml_diff>
--- a/p/content_by_grammar.xlsx
+++ b/p/content_by_grammar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adsv\private\books\language\ingush\Dahkilgov\github\dahkilgov\p\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{5E1E1EE6-2C6E-4BC3-8CB1-12CA48A869FE}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{59F09BE2-365F-433F-8B8D-FCF4FC9F7D1E}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2415" windowWidth="38640" windowHeight="21120" xr2:uid="{AC639D1C-64A7-45F6-9CFA-A1A688E9895B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="774" uniqueCount="320">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="786" uniqueCount="318">
   <si>
     <t>Причастие, несамостоятельное, настоящее время</t>
   </si>
@@ -47,9 +47,6 @@
     <t>Причастие, несамостоятельное, прошедшее время.</t>
   </si>
   <si>
-    <t>Деепричастие, настоящее время, отрицательная форма.</t>
-  </si>
-  <si>
     <t>Деепричастие, превращение в прилагательное.</t>
   </si>
   <si>
@@ -62,9 +59,6 @@
     <t>Прилагательное, множественное число, исключение для “доккха”.</t>
   </si>
   <si>
-    <t>Деепричастие, будущее время, отрицательная форма.</t>
-  </si>
-  <si>
     <t>Причастие, самостоятельное, прошедшее время.</t>
   </si>
   <si>
@@ -89,15 +83,9 @@
     <t>Морфология. Пространственные послелоги тIа, чу, ...</t>
   </si>
   <si>
-    <t>Наречие. Образ действия.</t>
-  </si>
-  <si>
     <t>Прилагательное. Общие сведения.</t>
   </si>
   <si>
-    <t>Наречие. Обозначение времени.</t>
-  </si>
-  <si>
     <t>Морфология. Отрицание.</t>
   </si>
   <si>
@@ -176,9 +164,6 @@
     <t>Существительное, классы, признаки, по которым можно определить класс.</t>
   </si>
   <si>
-    <t>Наречие, обозначение длительности.</t>
-  </si>
-  <si>
     <t>Деепричастие, изменение по классам.</t>
   </si>
   <si>
@@ -236,9 +221,6 @@
     <t>Существительное, падежи, склонение, 1-й тип, 2-й подтип.</t>
   </si>
   <si>
-    <t>Глагол, модальные глаголы.</t>
-  </si>
-  <si>
     <t>Существительное, падежи, склонение, 2-й тип, 1-й подтип.</t>
   </si>
   <si>
@@ -362,9 +344,6 @@
     <t>Фонетика. Несколько согласных в начале слова</t>
   </si>
   <si>
-    <t>Фонетика. Сочетание “рг” в середине слова, произношение.</t>
-  </si>
-  <si>
     <t>Синтаксис. Вопросительное предложение, слово «фуд».</t>
   </si>
   <si>
@@ -959,12 +938,6 @@
     <t>Глагол, вспомогательный глагол “де” - делать, сложные глаголы.</t>
   </si>
   <si>
-    <t>поменяться со 164, там шишша-кхоккха</t>
-  </si>
-  <si>
-    <t>поменяться с притчей про порядковые числительные</t>
-  </si>
-  <si>
     <t>Причастие, склонение по падежам.</t>
   </si>
   <si>
@@ -974,21 +947,12 @@
     <t>найти и заменить на Притчу с примером в отриц. форме</t>
   </si>
   <si>
-    <t>перенести отрицание ближе к концу, после ознакомления с терминами причастие, деепричастие, и т.д.</t>
-  </si>
-  <si>
     <t>перенести в начало ?</t>
   </si>
   <si>
     <t>Причастие, примеры разных форм причастий в разных временах.</t>
   </si>
   <si>
-    <t>заменить на модальную форму, Ахриева 184</t>
-  </si>
-  <si>
-    <t>заменить на совпадение формы деепричастия с причастием прошедшего времени</t>
-  </si>
-  <si>
     <t>Деепричастие, отрицательная форма.</t>
   </si>
   <si>
@@ -998,7 +962,37 @@
     <t>Деепричастие, соединительный оборот, окончания -е, -ий, -й.</t>
   </si>
   <si>
-    <t>заменить на примеры, переместить сразу после времен</t>
+    <t>Деепричастие, модальные обороты со вспомогательными глаголами.</t>
+  </si>
+  <si>
+    <t>Деепричастие, прошедшее время, совпадение формы с причастием.</t>
+  </si>
+  <si>
+    <t>Деепричастие, примеры.</t>
+  </si>
+  <si>
+    <t>Глагол, времена, будущее фактическое время, произношени “рг”.</t>
+  </si>
+  <si>
+    <t>164</t>
+  </si>
+  <si>
+    <t>111</t>
+  </si>
+  <si>
+    <t>143</t>
+  </si>
+  <si>
+    <t>поменять на притчу с примером масдара</t>
+  </si>
+  <si>
+    <t>Наречие, превосходная степень.</t>
+  </si>
+  <si>
+    <t>Наречие, обозначение времени.</t>
+  </si>
+  <si>
+    <t>Наречие, образ действия.</t>
   </si>
 </sst>
 </file>
@@ -1420,36 +1414,36 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>167</v>
+        <v>160</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>116</v>
+        <v>109</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="E1" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>168</v>
+        <v>161</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>105</v>
+        <v>99</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="E2" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
@@ -1457,16 +1451,16 @@
         <v>144</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>104</v>
+        <v>98</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="E3" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
@@ -1474,852 +1468,849 @@
         <v>105</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>267</v>
+        <v>260</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="E4" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>169</v>
+        <v>162</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>268</v>
+        <v>261</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="E5" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>170</v>
+        <v>163</v>
       </c>
       <c r="B6" s="1" t="s">
-        <v>106</v>
+        <v>100</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="E6" s="5" t="s">
-        <v>270</v>
+        <v>263</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A7" s="4">
-        <v>152</v>
+      <c r="A7" s="4" t="s">
+        <v>164</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>107</v>
+        <v>103</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
       <c r="E7" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A8" s="4" t="s">
-        <v>171</v>
+      <c r="A8" s="4">
+        <v>166</v>
       </c>
       <c r="B8" s="1" t="s">
+        <v>108</v>
+      </c>
+      <c r="C8" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="D8" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E8" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A9" s="4" t="s">
+        <v>165</v>
+      </c>
+      <c r="B9" s="1" t="s">
         <v>110</v>
       </c>
-      <c r="C8" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="D8" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E8" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="9" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A9" s="4">
-        <v>166</v>
-      </c>
-      <c r="B9" s="1" t="s">
-        <v>115</v>
-      </c>
       <c r="C9" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="E9" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>172</v>
+        <v>166</v>
       </c>
       <c r="B10" s="1" t="s">
-        <v>117</v>
+        <v>111</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E10" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>173</v>
+        <v>167</v>
       </c>
       <c r="B11" s="1" t="s">
-        <v>118</v>
+        <v>120</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E11" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>174</v>
+        <v>168</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>127</v>
+        <v>116</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>129</v>
+        <v>144</v>
       </c>
       <c r="E12" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A13" s="4" t="s">
-        <v>175</v>
+      <c r="A13" s="4">
+        <v>124</v>
       </c>
       <c r="B13" s="1" t="s">
-        <v>123</v>
+        <v>113</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E13" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4">
-        <v>124</v>
+        <v>116</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>120</v>
+        <v>114</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E14" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4">
-        <v>116</v>
+        <v>128</v>
       </c>
       <c r="B15" s="1" t="s">
+        <v>118</v>
+      </c>
+      <c r="C15" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D15" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E15" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A16" s="4" t="s">
+        <v>169</v>
+      </c>
+      <c r="B16" s="1" t="s">
+        <v>112</v>
+      </c>
+      <c r="C16" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D16" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E16" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="17" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A17" s="4" t="s">
+        <v>170</v>
+      </c>
+      <c r="B17" s="1" t="s">
+        <v>117</v>
+      </c>
+      <c r="C17" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D17" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E17" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="18" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A18" s="4" t="s">
+        <v>171</v>
+      </c>
+      <c r="B18" s="1" t="s">
+        <v>115</v>
+      </c>
+      <c r="C18" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D18" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E18" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="19" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A19" s="4" t="s">
+        <v>172</v>
+      </c>
+      <c r="B19" s="1" t="s">
+        <v>119</v>
+      </c>
+      <c r="C19" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="D19" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E19" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="20" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A20" s="4" t="s">
+        <v>173</v>
+      </c>
+      <c r="B20" s="1" t="s">
+        <v>104</v>
+      </c>
+      <c r="C20" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D20" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E20" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="21" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A21" s="4" t="s">
+        <v>174</v>
+      </c>
+      <c r="B21" s="1" t="s">
+        <v>105</v>
+      </c>
+      <c r="C21" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D21" s="3" t="s">
         <v>121</v>
       </c>
-      <c r="C15" s="3" t="s">
+      <c r="E21" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="22" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A22" s="4" t="s">
+        <v>176</v>
+      </c>
+      <c r="B22" s="1" t="s">
+        <v>15</v>
+      </c>
+      <c r="C22" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D22" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E22" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="23" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A23" s="4">
+        <v>165</v>
+      </c>
+      <c r="B23" s="1" t="s">
+        <v>95</v>
+      </c>
+      <c r="C23" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D23" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E23" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="24" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A24" s="4">
+        <v>137</v>
+      </c>
+      <c r="B24" s="1" t="s">
+        <v>264</v>
+      </c>
+      <c r="C24" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D24" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E24" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="25" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A25" s="4" t="s">
+        <v>177</v>
+      </c>
+      <c r="B25" s="1" t="s">
+        <v>13</v>
+      </c>
+      <c r="C25" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D25" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E25" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="26" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A26" s="4" t="s">
+        <v>178</v>
+      </c>
+      <c r="B26" s="1" t="s">
+        <v>265</v>
+      </c>
+      <c r="C26" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D26" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E26" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="27" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A27" s="4">
+        <v>138</v>
+      </c>
+      <c r="B27" s="1" t="s">
+        <v>66</v>
+      </c>
+      <c r="C27" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D27" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E27" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="28" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A28" s="4">
+        <v>117</v>
+      </c>
+      <c r="B28" s="1" t="s">
+        <v>266</v>
+      </c>
+      <c r="C28" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D28" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E28" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="29" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A29" s="4" t="s">
+        <v>179</v>
+      </c>
+      <c r="B29" s="1" t="s">
+        <v>268</v>
+      </c>
+      <c r="C29" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D29" s="3" t="s">
         <v>129</v>
       </c>
-      <c r="D15" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E15" t="s">
+      <c r="E29" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="30" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A30" s="4">
+        <v>147</v>
+      </c>
+      <c r="B30" s="1" t="s">
+        <v>267</v>
+      </c>
+      <c r="C30" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D30" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E30" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="31" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A31" s="4" t="s">
+        <v>180</v>
+      </c>
+      <c r="B31" s="1" t="s">
         <v>269</v>
       </c>
-    </row>
-    <row r="16" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A16" s="4">
-        <v>128</v>
-      </c>
-      <c r="B16" s="1" t="s">
-        <v>125</v>
-      </c>
-      <c r="C16" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D16" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E16" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="17" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A17" s="4" t="s">
-        <v>176</v>
-      </c>
-      <c r="B17" s="1" t="s">
-        <v>119</v>
-      </c>
-      <c r="C17" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D17" s="3" t="s">
+      <c r="C31" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="D31" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="E17" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="18" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>177</v>
-      </c>
-      <c r="B18" s="1" t="s">
+      <c r="E31" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="32" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A32" s="4" t="s">
+        <v>182</v>
+      </c>
+      <c r="B32" s="1" t="s">
+        <v>85</v>
+      </c>
+      <c r="C32" s="3" t="s">
         <v>124</v>
       </c>
-      <c r="C18" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D18" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E18" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="19" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A19" s="4" t="s">
-        <v>178</v>
-      </c>
-      <c r="B19" s="1" t="s">
-        <v>122</v>
-      </c>
-      <c r="C19" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D19" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E19" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="20" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A20" s="4" t="s">
-        <v>179</v>
-      </c>
-      <c r="B20" s="1" t="s">
-        <v>126</v>
-      </c>
-      <c r="C20" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="D20" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E20" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="21" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>180</v>
-      </c>
-      <c r="B21" s="1" t="s">
-        <v>111</v>
-      </c>
-      <c r="C21" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D21" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E21" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="22" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A22" s="4" t="s">
-        <v>181</v>
-      </c>
-      <c r="B22" s="1" t="s">
-        <v>112</v>
-      </c>
-      <c r="C22" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D22" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E22" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="23" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A23" s="4" t="s">
-        <v>183</v>
-      </c>
-      <c r="B23" s="1" t="s">
-        <v>19</v>
-      </c>
-      <c r="C23" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D23" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E23" t="s">
-        <v>269</v>
-      </c>
-      <c r="F23" t="s">
-        <v>311</v>
-      </c>
-    </row>
-    <row r="24" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A24" s="4">
-        <v>165</v>
-      </c>
-      <c r="B24" s="1" t="s">
-        <v>101</v>
-      </c>
-      <c r="C24" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D24" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E24" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="25" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A25" s="4">
-        <v>137</v>
-      </c>
-      <c r="B25" s="1" t="s">
-        <v>271</v>
-      </c>
-      <c r="C25" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D25" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E25" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="26" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A26" s="4" t="s">
-        <v>184</v>
-      </c>
-      <c r="B26" s="1" t="s">
-        <v>15</v>
-      </c>
-      <c r="C26" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D26" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E26" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="27" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A27" s="4" t="s">
-        <v>185</v>
-      </c>
-      <c r="B27" s="1" t="s">
-        <v>272</v>
-      </c>
-      <c r="C27" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D27" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E27" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="28" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A28" s="4">
-        <v>138</v>
-      </c>
-      <c r="B28" s="1" t="s">
-        <v>72</v>
-      </c>
-      <c r="C28" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D28" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E28" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="29" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A29" s="4">
-        <v>117</v>
-      </c>
-      <c r="B29" s="1" t="s">
-        <v>273</v>
-      </c>
-      <c r="C29" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D29" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E29" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="30" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A30" s="4" t="s">
-        <v>186</v>
-      </c>
-      <c r="B30" s="1" t="s">
-        <v>275</v>
-      </c>
-      <c r="C30" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D30" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E30" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="31" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A31" s="4">
-        <v>147</v>
-      </c>
-      <c r="B31" s="1" t="s">
-        <v>274</v>
-      </c>
-      <c r="C31" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="D31" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E31" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="32" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A32" s="4" t="s">
-        <v>187</v>
-      </c>
-      <c r="B32" s="1" t="s">
-        <v>276</v>
-      </c>
-      <c r="C32" s="3" t="s">
-        <v>130</v>
-      </c>
       <c r="D32" s="3" t="s">
-        <v>138</v>
+        <v>144</v>
       </c>
       <c r="E32" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>189</v>
+        <v>183</v>
       </c>
       <c r="B33" s="1" t="s">
-        <v>91</v>
+        <v>35</v>
       </c>
       <c r="C33" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D33" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E33" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A34" s="4" t="s">
-        <v>190</v>
+      <c r="A34" s="4">
+        <v>114</v>
       </c>
       <c r="B34" s="1" t="s">
-        <v>39</v>
+        <v>40</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E34" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A35" s="4">
-        <v>114</v>
+      <c r="A35" s="4" t="s">
+        <v>184</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>44</v>
+        <v>88</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E35" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="36" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>191</v>
+        <v>185</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>94</v>
+        <v>9</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E36" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="37" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>192</v>
+        <v>186</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>11</v>
+        <v>270</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E37" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="38" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A38" s="4" t="s">
-        <v>193</v>
+      <c r="A38" s="4">
+        <v>134</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>277</v>
+        <v>91</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E38" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="39" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A39" s="4">
-        <v>134</v>
+        <v>106</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>97</v>
+        <v>37</v>
       </c>
       <c r="C39" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D39" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E39" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="40" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A40" s="4">
-        <v>106</v>
+      <c r="A40" s="4" t="s">
+        <v>181</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>41</v>
+        <v>271</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E40" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="41" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>278</v>
+        <v>86</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E41" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="42" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>194</v>
+        <v>189</v>
       </c>
       <c r="B42" s="1" t="s">
-        <v>92</v>
+        <v>30</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E42" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="43" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>196</v>
+        <v>190</v>
       </c>
       <c r="B43" s="1" t="s">
-        <v>34</v>
+        <v>28</v>
       </c>
       <c r="C43" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="D43" s="3" t="s">
         <v>131</v>
       </c>
-      <c r="D43" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="E43" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="44" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>197</v>
+        <v>191</v>
       </c>
       <c r="B44" s="1" t="s">
-        <v>32</v>
+        <v>16</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E44" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="45" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>198</v>
+        <v>192</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>20</v>
+        <v>56</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E45" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="46" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>199</v>
+        <v>193</v>
       </c>
       <c r="B46" s="1" t="s">
-        <v>61</v>
+        <v>29</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E46" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="47" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>200</v>
+        <v>194</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>33</v>
+        <v>89</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D47" s="3" t="s">
+        <v>135</v>
+      </c>
+      <c r="E47" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A48" s="4">
         <v>141</v>
       </c>
-      <c r="E47" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="48" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A48" s="4" t="s">
-        <v>201</v>
-      </c>
       <c r="B48" s="1" t="s">
-        <v>95</v>
+        <v>90</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E48" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="49" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A49" s="4">
-        <v>141</v>
+        <v>167</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>96</v>
+        <v>75</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E49" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="50" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A50" s="4">
-        <v>167</v>
+        <v>155</v>
       </c>
       <c r="B50" s="1" t="s">
-        <v>81</v>
+        <v>72</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E50" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="51" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A51" s="4">
-        <v>155</v>
+        <v>170</v>
       </c>
       <c r="B51" s="1" t="s">
-        <v>78</v>
+        <v>76</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E51" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="52" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A52" s="4">
-        <v>170</v>
+        <v>154</v>
       </c>
       <c r="B52" s="1" t="s">
-        <v>82</v>
+        <v>87</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E52" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="53" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A53" s="4">
-        <v>154</v>
+      <c r="A53" s="4" t="s">
+        <v>188</v>
       </c>
       <c r="B53" s="1" t="s">
-        <v>93</v>
+        <v>57</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E53" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="54" spans="1:5" x14ac:dyDescent="0.3">
@@ -2327,750 +2318,747 @@
         <v>195</v>
       </c>
       <c r="B54" s="1" t="s">
-        <v>62</v>
+        <v>58</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E54" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="55" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>202</v>
+        <v>196</v>
       </c>
       <c r="B55" s="1" t="s">
-        <v>63</v>
+        <v>59</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E55" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="56" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>203</v>
+        <v>197</v>
       </c>
       <c r="B56" s="1" t="s">
-        <v>64</v>
+        <v>272</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E56" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="57" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>204</v>
+        <v>198</v>
       </c>
       <c r="B57" s="1" t="s">
-        <v>279</v>
+        <v>60</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E57" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="58" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A58" s="4" t="s">
-        <v>205</v>
+      <c r="A58" s="4">
+        <v>100</v>
       </c>
       <c r="B58" s="1" t="s">
-        <v>66</v>
+        <v>61</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E58" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="59" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A59" s="4">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="B59" s="1" t="s">
-        <v>67</v>
+        <v>273</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="E59" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="60" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A60" s="4">
-        <v>101</v>
+      <c r="A60" s="4" t="s">
+        <v>233</v>
       </c>
       <c r="B60" s="1" t="s">
-        <v>280</v>
+        <v>274</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="E60" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="61" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>240</v>
+        <v>276</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>281</v>
+        <v>277</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E61" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="62" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>283</v>
+        <v>199</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>284</v>
+        <v>14</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>160</v>
+        <v>144</v>
       </c>
       <c r="E62" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="63" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>206</v>
+        <v>200</v>
       </c>
       <c r="B63" s="1" t="s">
-        <v>17</v>
+        <v>33</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E63" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="64" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
+        <v>201</v>
+      </c>
+      <c r="B64" s="1" t="s">
+        <v>34</v>
+      </c>
+      <c r="C64" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D64" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E64" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="65" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A65" s="4">
+        <v>142</v>
+      </c>
+      <c r="B65" s="1" t="s">
+        <v>65</v>
+      </c>
+      <c r="C65" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D65" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E65" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="66" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A66" s="4" t="s">
+        <v>202</v>
+      </c>
+      <c r="B66" s="1" t="s">
+        <v>278</v>
+      </c>
+      <c r="C66" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D66" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E66" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="67" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A67" s="4">
+        <v>126</v>
+      </c>
+      <c r="B67" s="1" t="s">
+        <v>63</v>
+      </c>
+      <c r="C67" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D67" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="E67" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="68" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A68" s="4" t="s">
+        <v>203</v>
+      </c>
+      <c r="B68" s="1" t="s">
+        <v>48</v>
+      </c>
+      <c r="C68" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D68" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="E68" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="69" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A69" s="4" t="s">
+        <v>204</v>
+      </c>
+      <c r="B69" s="1" t="s">
+        <v>279</v>
+      </c>
+      <c r="C69" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D69" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="E69" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="70" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A70" s="4">
+        <v>151</v>
+      </c>
+      <c r="B70" s="1" t="s">
+        <v>92</v>
+      </c>
+      <c r="C70" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D70" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="E70" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="71" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A71" s="4" t="s">
+        <v>205</v>
+      </c>
+      <c r="B71" s="1" t="s">
+        <v>53</v>
+      </c>
+      <c r="C71" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D71" s="3" t="s">
+        <v>129</v>
+      </c>
+      <c r="E71" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="72" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A72" s="4">
+        <v>149</v>
+      </c>
+      <c r="B72" s="1" t="s">
+        <v>5</v>
+      </c>
+      <c r="C72" s="3" t="s">
+        <v>125</v>
+      </c>
+      <c r="D72" s="3" t="s">
+        <v>130</v>
+      </c>
+      <c r="E72" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="73" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A73" s="4" t="s">
+        <v>206</v>
+      </c>
+      <c r="B73" s="1" t="s">
+        <v>10</v>
+      </c>
+      <c r="C73" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D73" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E73" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="74" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A74" s="4">
+        <v>107</v>
+      </c>
+      <c r="B74" s="1" t="s">
+        <v>281</v>
+      </c>
+      <c r="C74" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D74" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E74" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="75" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A75" s="4" t="s">
+        <v>313</v>
+      </c>
+      <c r="B75" s="1" t="s">
+        <v>282</v>
+      </c>
+      <c r="C75" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D75" s="3" t="s">
+        <v>122</v>
+      </c>
+      <c r="E75" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="76" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A76" s="4" t="s">
         <v>207</v>
       </c>
-      <c r="B64" s="1" t="s">
-        <v>37</v>
-      </c>
-      <c r="C64" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D64" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E64" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="65" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A65" s="4" t="s">
+      <c r="B76" s="1" t="s">
+        <v>283</v>
+      </c>
+      <c r="C76" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D76" s="3" t="s">
+        <v>123</v>
+      </c>
+      <c r="E76" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="77" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A77" s="4" t="s">
+        <v>311</v>
+      </c>
+      <c r="B77" s="1" t="s">
+        <v>280</v>
+      </c>
+      <c r="C77" s="3" t="s">
+        <v>126</v>
+      </c>
+      <c r="D77" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E77" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="78" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A78" s="4" t="s">
         <v>208</v>
       </c>
-      <c r="B65" s="1" t="s">
-        <v>38</v>
-      </c>
-      <c r="C65" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D65" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E65" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="66" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A66" s="4">
-        <v>142</v>
-      </c>
-      <c r="B66" s="1" t="s">
-        <v>71</v>
-      </c>
-      <c r="C66" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D66" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E66" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="67" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A67" s="4" t="s">
+      <c r="B78" s="1" t="s">
+        <v>7</v>
+      </c>
+      <c r="C78" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D78" s="3" t="s">
+        <v>144</v>
+      </c>
+      <c r="E78" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="79" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A79" s="4" t="s">
         <v>209</v>
       </c>
-      <c r="B67" s="1" t="s">
-        <v>285</v>
-      </c>
-      <c r="C67" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D67" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E67" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="68" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A68" s="4">
-        <v>126</v>
-      </c>
-      <c r="B68" s="1" t="s">
-        <v>69</v>
-      </c>
-      <c r="C68" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D68" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="E68" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="69" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A69" s="4" t="s">
+      <c r="B79" s="1" t="s">
+        <v>32</v>
+      </c>
+      <c r="C79" s="3" t="s">
+        <v>127</v>
+      </c>
+      <c r="D79" s="3" t="s">
+        <v>121</v>
+      </c>
+      <c r="E79" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="80" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A80" s="4" t="s">
         <v>210</v>
       </c>
-      <c r="B69" s="1" t="s">
-        <v>53</v>
-      </c>
-      <c r="C69" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D69" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="E69" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="70" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A70" s="4" t="s">
-        <v>211</v>
-      </c>
-      <c r="B70" s="1" t="s">
-        <v>286</v>
-      </c>
-      <c r="C70" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D70" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E70" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="71" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A71" s="4">
-        <v>151</v>
-      </c>
-      <c r="B71" s="1" t="s">
-        <v>98</v>
-      </c>
-      <c r="C71" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D71" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="E71" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="72" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A72" s="4" t="s">
-        <v>212</v>
-      </c>
-      <c r="B72" s="1" t="s">
-        <v>58</v>
-      </c>
-      <c r="C72" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D72" s="3" t="s">
-        <v>136</v>
-      </c>
-      <c r="E72" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="73" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A73" s="4">
-        <v>149</v>
-      </c>
-      <c r="B73" s="1" t="s">
-        <v>6</v>
-      </c>
-      <c r="C73" s="3" t="s">
-        <v>132</v>
-      </c>
-      <c r="D73" s="3" t="s">
-        <v>137</v>
-      </c>
-      <c r="E73" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="74" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A74" s="4" t="s">
-        <v>213</v>
-      </c>
-      <c r="B74" s="1" t="s">
-        <v>12</v>
-      </c>
-      <c r="C74" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E74" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="75" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A75" s="4">
-        <v>107</v>
-      </c>
-      <c r="B75" s="1" t="s">
-        <v>288</v>
-      </c>
-      <c r="C75" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D75" s="3" t="s">
-        <v>128</v>
-      </c>
-      <c r="E75" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="76" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A76" s="4">
-        <v>164</v>
-      </c>
-      <c r="B76" s="1" t="s">
-        <v>289</v>
-      </c>
-      <c r="C76" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D76" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="E76" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="77" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A77" s="4" t="s">
-        <v>214</v>
-      </c>
-      <c r="B77" s="1" t="s">
-        <v>290</v>
-      </c>
-      <c r="C77" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D77" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E77" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="78" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A78" s="4">
-        <v>111</v>
-      </c>
-      <c r="B78" s="1" t="s">
-        <v>287</v>
-      </c>
-      <c r="C78" s="3" t="s">
-        <v>133</v>
-      </c>
-      <c r="D78" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="E78" t="s">
-        <v>269</v>
-      </c>
-      <c r="F78" t="s">
-        <v>306</v>
-      </c>
-    </row>
-    <row r="79" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A79" s="4" t="s">
-        <v>215</v>
-      </c>
-      <c r="B79" s="1" t="s">
-        <v>9</v>
-      </c>
-      <c r="C79" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="D79" s="3" t="s">
-        <v>151</v>
-      </c>
-      <c r="E79" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="80" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A80" s="4" t="s">
-        <v>216</v>
-      </c>
       <c r="B80" s="1" t="s">
-        <v>36</v>
+        <v>17</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E80" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="81" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>217</v>
+        <v>211</v>
       </c>
       <c r="B81" s="1" t="s">
-        <v>21</v>
+        <v>50</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E81" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="82" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>218</v>
+        <v>212</v>
       </c>
       <c r="B82" s="1" t="s">
-        <v>55</v>
+        <v>19</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E82" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="83" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>219</v>
+        <v>275</v>
       </c>
       <c r="B83" s="1" t="s">
-        <v>23</v>
+        <v>20</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E83" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="84" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>282</v>
+        <v>214</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E84" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="85" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A85" s="4" t="s">
-        <v>221</v>
+      <c r="A85" s="4">
+        <v>158</v>
       </c>
       <c r="B85" s="1" t="s">
-        <v>28</v>
+        <v>74</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E85" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="86" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A86" s="4">
-        <v>158</v>
+        <v>140</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>80</v>
+        <v>68</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E86" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="87" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A87" s="4">
-        <v>140</v>
+        <v>112</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>74</v>
+        <v>4</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>135</v>
+        <v>144</v>
       </c>
       <c r="E87" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="88" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A88" s="4">
-        <v>112</v>
+      <c r="A88" s="4" t="s">
+        <v>215</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>5</v>
+        <v>31</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E88" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="89" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>222</v>
+        <v>216</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>35</v>
+        <v>78</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E89" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="90" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>223</v>
+        <v>217</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>84</v>
+        <v>21</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E90" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="91" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A91" s="4" t="s">
-        <v>224</v>
+      <c r="A91" s="4">
+        <v>108</v>
       </c>
       <c r="B91" s="1" t="s">
+        <v>82</v>
+      </c>
+      <c r="C91" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D91" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E91" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
+      <c r="A92" s="4" t="s">
+        <v>218</v>
+      </c>
+      <c r="B92" s="1" t="s">
         <v>25</v>
       </c>
-      <c r="C91" s="3" t="s">
-        <v>135</v>
-      </c>
-      <c r="D91" s="3" t="s">
-        <v>130</v>
-      </c>
-      <c r="E91" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="92" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A92" s="4">
-        <v>108</v>
-      </c>
-      <c r="B92" s="1" t="s">
-        <v>88</v>
-      </c>
       <c r="C92" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E92" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="93" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A93" s="4" t="s">
-        <v>225</v>
+      <c r="A93" s="4">
+        <v>110</v>
       </c>
       <c r="B93" s="1" t="s">
-        <v>29</v>
+        <v>38</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E93" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="94" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A94" s="4">
-        <v>110</v>
+        <v>152</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>42</v>
+        <v>310</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E94" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="95" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>226</v>
+        <v>219</v>
       </c>
       <c r="B95" s="1" t="s">
-        <v>48</v>
+        <v>43</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E95" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="96" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>227</v>
+        <v>220</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>26</v>
+        <v>22</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E96" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>228</v>
+        <v>221</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>40</v>
+        <v>36</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E97" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
@@ -3078,33 +3066,33 @@
         <v>168</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>83</v>
+        <v>77</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E98" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>229</v>
+        <v>222</v>
       </c>
       <c r="B99" s="1" t="s">
-        <v>49</v>
+        <v>44</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E99" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
@@ -3112,67 +3100,67 @@
         <v>104</v>
       </c>
       <c r="B100" s="1" t="s">
-        <v>89</v>
+        <v>83</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E100" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A101" s="4" t="s">
-        <v>231</v>
+        <v>224</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>47</v>
+        <v>42</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E101" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A102" s="4" t="s">
-        <v>230</v>
+        <v>223</v>
       </c>
       <c r="B102" s="1" t="s">
-        <v>90</v>
+        <v>84</v>
       </c>
       <c r="C102" s="3" t="s">
+        <v>128</v>
+      </c>
+      <c r="D102" s="3" t="s">
         <v>135</v>
       </c>
-      <c r="D102" s="3" t="s">
-        <v>141</v>
-      </c>
       <c r="E102" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>232</v>
+        <v>225</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>54</v>
+        <v>49</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>142</v>
+        <v>136</v>
       </c>
       <c r="E103" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
@@ -3180,16 +3168,16 @@
         <v>153</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>77</v>
+        <v>71</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>143</v>
+        <v>137</v>
       </c>
       <c r="E104" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
@@ -3197,16 +3185,16 @@
         <v>146</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>76</v>
+        <v>70</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>144</v>
+        <v>138</v>
       </c>
       <c r="E105" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="106" spans="1:6" x14ac:dyDescent="0.3">
@@ -3214,16 +3202,16 @@
         <v>115</v>
       </c>
       <c r="B106" s="1" t="s">
-        <v>87</v>
+        <v>81</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>145</v>
+        <v>139</v>
       </c>
       <c r="E106" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -3231,16 +3219,16 @@
         <v>139</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>73</v>
+        <v>67</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>146</v>
+        <v>140</v>
       </c>
       <c r="E107" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
@@ -3248,33 +3236,33 @@
         <v>136</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>291</v>
+        <v>284</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>147</v>
+        <v>141</v>
       </c>
       <c r="E108" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A109" s="4" t="s">
-        <v>233</v>
+        <v>226</v>
       </c>
       <c r="B109" s="1" t="s">
-        <v>85</v>
+        <v>79</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>148</v>
+        <v>142</v>
       </c>
       <c r="E109" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
@@ -3282,158 +3270,158 @@
         <v>130</v>
       </c>
       <c r="B110" s="1" t="s">
-        <v>70</v>
+        <v>64</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>149</v>
+        <v>143</v>
       </c>
       <c r="E110" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
-        <v>242</v>
+        <v>235</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>51</v>
+        <v>46</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="E111" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A112" s="4" t="s">
-        <v>235</v>
+        <v>228</v>
       </c>
       <c r="B112" s="1" t="s">
-        <v>293</v>
+        <v>286</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>156</v>
+        <v>150</v>
       </c>
       <c r="E112" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F112" s="5"/>
     </row>
     <row r="113" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A113" s="4" t="s">
-        <v>238</v>
+        <v>231</v>
       </c>
       <c r="B113" s="1" t="s">
-        <v>297</v>
+        <v>290</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>157</v>
+        <v>151</v>
       </c>
       <c r="E113" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F113" s="5"/>
     </row>
     <row r="114" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A114" s="4" t="s">
-        <v>261</v>
+        <v>254</v>
       </c>
       <c r="B114" s="1" t="s">
-        <v>296</v>
+        <v>289</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>158</v>
+        <v>152</v>
       </c>
       <c r="E114" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F114" s="5"/>
     </row>
     <row r="115" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A115" s="4" t="s">
-        <v>234</v>
+        <v>227</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>295</v>
+        <v>288</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>159</v>
+        <v>147</v>
       </c>
       <c r="E115" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F115" s="5"/>
     </row>
     <row r="116" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A116" s="4" t="s">
-        <v>237</v>
+        <v>230</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>298</v>
+        <v>291</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="E116" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F116" s="5"/>
     </row>
     <row r="117" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A117" s="4" t="s">
-        <v>220</v>
+        <v>213</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>294</v>
+        <v>287</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>160</v>
+        <v>148</v>
       </c>
       <c r="E117" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F117" s="5"/>
     </row>
     <row r="118" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A118" s="4" t="s">
-        <v>236</v>
+        <v>229</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>292</v>
+        <v>285</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="E118" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
       <c r="F118" s="5"/>
     </row>
@@ -3442,33 +3430,33 @@
         <v>131</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>305</v>
+        <v>298</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>161</v>
+        <v>155</v>
       </c>
       <c r="E119" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="120" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A120" s="4" t="s">
-        <v>299</v>
+        <v>292</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>303</v>
+        <v>296</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>162</v>
+        <v>156</v>
       </c>
       <c r="E120" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="121" spans="1:6" x14ac:dyDescent="0.3">
@@ -3476,345 +3464,345 @@
         <v>148</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>304</v>
+        <v>297</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>163</v>
+        <v>157</v>
       </c>
       <c r="E121" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="122" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A122" s="4" t="s">
-        <v>241</v>
+        <v>236</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>65</v>
+        <v>27</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>164</v>
+        <v>158</v>
       </c>
       <c r="E122" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="123" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A123" s="4" t="s">
-        <v>243</v>
+      <c r="A123" s="4">
+        <v>159</v>
       </c>
       <c r="B123" s="1" t="s">
-        <v>31</v>
+        <v>80</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>165</v>
+        <v>159</v>
       </c>
       <c r="E123" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="124" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A124" s="4">
-        <v>159</v>
+        <v>125</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>86</v>
+        <v>146</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>166</v>
+        <v>144</v>
       </c>
       <c r="E124" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="125" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A125" s="4">
-        <v>125</v>
+      <c r="A125" s="4" t="s">
+        <v>312</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>153</v>
+        <v>145</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>136</v>
+        <v>129</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E125" t="s">
-        <v>269</v>
+        <v>262</v>
+      </c>
+      <c r="F125" t="s">
+        <v>314</v>
       </c>
     </row>
     <row r="126" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A126" s="4">
-        <v>143</v>
+      <c r="A126" s="4" t="s">
+        <v>237</v>
       </c>
       <c r="B126" s="1" t="s">
-        <v>152</v>
+        <v>47</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>128</v>
+        <v>144</v>
       </c>
       <c r="E126" t="s">
-        <v>269</v>
-      </c>
-      <c r="F126" t="s">
-        <v>307</v>
+        <v>262</v>
       </c>
     </row>
     <row r="127" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A127" s="4" t="s">
-        <v>244</v>
+        <v>238</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>52</v>
+        <v>0</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E127" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="128" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A128" s="4" t="s">
-        <v>245</v>
+      <c r="A128" s="4">
+        <v>157</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>0</v>
+        <v>73</v>
       </c>
       <c r="C128" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D128" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E128" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="129" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A129" s="4">
-        <v>157</v>
+      <c r="A129" s="4" t="s">
+        <v>239</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>79</v>
+        <v>1</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>129</v>
+        <v>123</v>
       </c>
       <c r="E129" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="130" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A130" s="4" t="s">
-        <v>246</v>
+      <c r="A130" s="4">
+        <v>109</v>
       </c>
       <c r="B130" s="1" t="s">
-        <v>1</v>
+        <v>3</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D130" s="3" t="s">
+        <v>124</v>
+      </c>
+      <c r="E130" t="s">
+        <v>262</v>
+      </c>
+    </row>
+    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
+      <c r="A131" s="4" t="s">
+        <v>240</v>
+      </c>
+      <c r="B131" s="1" t="s">
+        <v>55</v>
+      </c>
+      <c r="C131" s="3" t="s">
         <v>130</v>
       </c>
-      <c r="E130" t="s">
-        <v>269</v>
-      </c>
-    </row>
-    <row r="131" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A131" s="4">
-        <v>109</v>
-      </c>
-      <c r="B131" s="1" t="s">
-        <v>4</v>
-      </c>
-      <c r="C131" s="3" t="s">
-        <v>137</v>
-      </c>
       <c r="D131" s="3" t="s">
-        <v>131</v>
+        <v>125</v>
       </c>
       <c r="E131" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="132" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A132" s="4" t="s">
-        <v>247</v>
+      <c r="A132" s="4">
+        <v>161</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>60</v>
+        <v>6</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E132" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="133" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A133" s="4">
-        <v>161</v>
+      <c r="A133" s="4" t="s">
+        <v>241</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>8</v>
+        <v>303</v>
       </c>
       <c r="C133" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D133" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E133" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="134" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A134" s="4" t="s">
-        <v>248</v>
+        <v>175</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>313</v>
+        <v>300</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>134</v>
+        <v>128</v>
       </c>
       <c r="E134" t="s">
-        <v>269</v>
+        <v>262</v>
+      </c>
+      <c r="F134" t="s">
+        <v>301</v>
       </c>
     </row>
     <row r="135" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A135" s="4" t="s">
-        <v>182</v>
+      <c r="A135" s="4">
+        <v>121</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>309</v>
+        <v>299</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>137</v>
+        <v>130</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E135" t="s">
-        <v>269</v>
-      </c>
-      <c r="F135" t="s">
-        <v>310</v>
+        <v>262</v>
       </c>
     </row>
     <row r="136" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A136" s="4">
-        <v>121</v>
+      <c r="A136" s="4" t="s">
+        <v>242</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>308</v>
+        <v>18</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>136</v>
+        <v>144</v>
       </c>
       <c r="E136" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="137" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A137" s="4" t="s">
-        <v>249</v>
+        <v>243</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>22</v>
+        <v>54</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>151</v>
+        <v>121</v>
       </c>
       <c r="E137" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="138" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A138" s="4" t="s">
-        <v>250</v>
+      <c r="A138" s="4">
+        <v>113</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>59</v>
+        <v>39</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>128</v>
+        <v>122</v>
       </c>
       <c r="E138" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="139" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A139" s="4" t="s">
-        <v>251</v>
+      <c r="A139" s="4">
+        <v>102</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>2</v>
+        <v>62</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>129</v>
-      </c>
-      <c r="F139" t="s">
-        <v>315</v>
+        <v>123</v>
+      </c>
+      <c r="E139" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="140" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A140" s="4">
-        <v>113</v>
+      <c r="A140" s="4" t="s">
+        <v>244</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>43</v>
+        <v>308</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>130</v>
+        <v>124</v>
       </c>
       <c r="E140" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="141" spans="1:6" x14ac:dyDescent="0.3">
@@ -3822,101 +3810,101 @@
         <v>150</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>7</v>
+        <v>309</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>131</v>
-      </c>
-      <c r="F141" t="s">
-        <v>314</v>
+        <v>125</v>
+      </c>
+      <c r="E141" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="142" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A142" s="4">
-        <v>102</v>
+        <v>156</v>
       </c>
       <c r="B142" s="1" t="s">
-        <v>68</v>
+        <v>304</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>132</v>
+        <v>126</v>
       </c>
       <c r="E142" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="143" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A143" s="4">
-        <v>156</v>
+        <v>123</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>316</v>
+        <v>41</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>133</v>
+        <v>127</v>
       </c>
       <c r="E143" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="144" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A144" s="4">
-        <v>123</v>
+      <c r="A144" s="4" t="s">
+        <v>245</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>46</v>
+        <v>2</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="F144" t="s">
-        <v>319</v>
+        <v>128</v>
+      </c>
+      <c r="E144" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="145" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A145" s="4" t="s">
-        <v>252</v>
+      <c r="A145" s="4">
+        <v>145</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>3</v>
+        <v>69</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>135</v>
+        <v>129</v>
       </c>
       <c r="E145" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="146" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A146" s="4">
-        <v>145</v>
+      <c r="A146" s="4" t="s">
+        <v>234</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>75</v>
+        <v>307</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>136</v>
+        <v>130</v>
       </c>
       <c r="E146" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="147" spans="1:5" x14ac:dyDescent="0.3">
@@ -3924,16 +3912,16 @@
         <v>135</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>317</v>
+        <v>305</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>137</v>
+        <v>131</v>
       </c>
       <c r="E147" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="148" spans="1:5" x14ac:dyDescent="0.3">
@@ -3941,16 +3929,16 @@
         <v>133</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>318</v>
+        <v>306</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>138</v>
+        <v>132</v>
       </c>
       <c r="E148" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="149" spans="1:5" x14ac:dyDescent="0.3">
@@ -3958,16 +3946,16 @@
         <v>118</v>
       </c>
       <c r="B149" s="1" t="s">
-        <v>302</v>
+        <v>295</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>139</v>
+        <v>133</v>
       </c>
       <c r="E149" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="150" spans="1:5" x14ac:dyDescent="0.3">
@@ -3975,16 +3963,16 @@
         <v>160</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>300</v>
+        <v>293</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>140</v>
+        <v>134</v>
       </c>
       <c r="E150" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="151" spans="1:5" x14ac:dyDescent="0.3">
@@ -3992,128 +3980,152 @@
         <v>119</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>301</v>
+        <v>294</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>138</v>
+        <v>131</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>141</v>
+        <v>135</v>
       </c>
       <c r="E151" t="s">
-        <v>269</v>
+        <v>262</v>
       </c>
     </row>
     <row r="152" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A152" s="4" t="s">
-        <v>253</v>
+        <v>246</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>10</v>
+        <v>8</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
+      </c>
+      <c r="E152" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="153" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A153" s="4" t="s">
-        <v>254</v>
+        <v>247</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>18</v>
+        <v>316</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
+      </c>
+      <c r="E153" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="154" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A154" s="4" t="s">
-        <v>255</v>
+        <v>248</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>16</v>
+        <v>317</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>129</v>
+        <v>122</v>
+      </c>
+      <c r="E154" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="155" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A155" s="4" t="s">
-        <v>256</v>
+        <v>249</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>14</v>
+        <v>12</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>130</v>
+        <v>123</v>
+      </c>
+      <c r="E155" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="156" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A156" s="4" t="s">
-        <v>257</v>
+        <v>250</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>13</v>
+        <v>11</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
+      </c>
+      <c r="E156" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="157" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A157" s="4" t="s">
-        <v>258</v>
+        <v>251</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
+      </c>
+      <c r="E157" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="158" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A158" s="4" t="s">
-        <v>259</v>
+        <v>252</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>27</v>
+        <v>23</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
+      </c>
+      <c r="E158" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="159" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A159" s="4" t="s">
-        <v>260</v>
+        <v>253</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>57</v>
+        <v>52</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
+      </c>
+      <c r="E159" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="160" spans="1:5" x14ac:dyDescent="0.3">
@@ -4121,92 +4133,101 @@
         <v>120</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>45</v>
+        <v>315</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>139</v>
+        <v>132</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>135</v>
+        <v>128</v>
+      </c>
+      <c r="E160" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="161" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A161" s="4" t="s">
-        <v>239</v>
+        <v>232</v>
       </c>
       <c r="B161" s="1" t="s">
-        <v>30</v>
+        <v>26</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
+      </c>
+      <c r="E161" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="162" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
-        <v>262</v>
+        <v>255</v>
       </c>
       <c r="B162" s="1" t="s">
-        <v>50</v>
+        <v>45</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>140</v>
+        <v>133</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
+      </c>
+      <c r="E162" t="s">
+        <v>262</v>
       </c>
     </row>
     <row r="163" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
-        <v>263</v>
+        <v>256</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>114</v>
+        <v>107</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
       <c r="F163" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="164" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
-        <v>264</v>
+        <v>257</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>109</v>
+        <v>102</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>128</v>
+        <v>121</v>
       </c>
       <c r="F164" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="165" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A165" s="4" t="s">
-        <v>265</v>
+        <v>258</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>108</v>
+        <v>101</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>129</v>
+        <v>122</v>
       </c>
       <c r="F165" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="166" spans="1:6" x14ac:dyDescent="0.3">
@@ -4214,16 +4235,16 @@
         <v>132</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>103</v>
+        <v>97</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>130</v>
+        <v>123</v>
       </c>
       <c r="F166" t="s">
-        <v>312</v>
+        <v>302</v>
       </c>
     </row>
     <row r="167" spans="1:6" x14ac:dyDescent="0.3">
@@ -4231,13 +4252,13 @@
         <v>129</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>100</v>
+        <v>94</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>131</v>
+        <v>124</v>
       </c>
     </row>
     <row r="168" spans="1:6" x14ac:dyDescent="0.3">
@@ -4245,13 +4266,13 @@
         <v>127</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>99</v>
+        <v>93</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>132</v>
+        <v>125</v>
       </c>
     </row>
     <row r="169" spans="1:6" x14ac:dyDescent="0.3">
@@ -4259,13 +4280,13 @@
         <v>169</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>113</v>
+        <v>106</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>133</v>
+        <v>126</v>
       </c>
     </row>
     <row r="170" spans="1:6" x14ac:dyDescent="0.3">
@@ -4273,13 +4294,13 @@
         <v>122</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>102</v>
+        <v>96</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>141</v>
+        <v>134</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>134</v>
+        <v>127</v>
       </c>
     </row>
     <row r="171" spans="1:6" x14ac:dyDescent="0.3">
@@ -4287,13 +4308,13 @@
         <v>171</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>266</v>
+        <v>259</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>142</v>
+        <v>135</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>151</v>
+        <v>144</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
fixes for layout, palochka's
</commit_message>
<xml_diff>
--- a/p/content_by_grammar.xlsx
+++ b/p/content_by_grammar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adsv\private\books\language\ingush\Dahkilgov\github\dahkilgov\p\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{95F51437-6170-42F7-95AE-331AF76B3E75}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{A212BEE3-F116-4F07-83AE-65C051F8C76B}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="-108" yWindow="-108" windowWidth="23256" windowHeight="13896" xr2:uid="{AC639D1C-64A7-45F6-9CFA-A1A688E9895B}"/>
   </bookViews>
@@ -39,7 +39,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="644" uniqueCount="316">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="621" uniqueCount="316">
   <si>
     <t>Причастие, несамостоятельное, прошедшее время.</t>
   </si>
@@ -227,9 +227,6 @@
     <t>Прилагательное, качественное, самостоятельное.</t>
   </si>
   <si>
-    <t>Морфология. Составные послелоги, г1олла.</t>
-  </si>
-  <si>
     <t>Глагол, времена, употребление настоящего времени в значении будущего и прошедшего.</t>
   </si>
   <si>
@@ -797,9 +794,6 @@
     <t>Фонетика. Дифтонги оа, иэ, уо, ов, ув.</t>
   </si>
   <si>
-    <t>+</t>
-  </si>
-  <si>
     <t>Морфология. Составные слова, фразеологические обороты.</t>
   </si>
   <si>
@@ -932,9 +926,6 @@
     <t>Деепричастие, примеры.</t>
   </si>
   <si>
-    <t>Глагол, времена, будущее фактическое время, произношени “рг”.</t>
-  </si>
-  <si>
     <t>164</t>
   </si>
   <si>
@@ -987,6 +978,15 @@
   </si>
   <si>
     <t>Существительное, падежи, склонение, 1-й тип, примеры.</t>
+  </si>
+  <si>
+    <t>найти и заменить на Притчу с примером</t>
+  </si>
+  <si>
+    <t>Глагол, времена, будущее фактическое время, произношение “рг”.</t>
+  </si>
+  <si>
+    <t>Морфология. Составные послелоги, гӀолла.</t>
   </si>
 </sst>
 </file>
@@ -1408,1472 +1408,1405 @@
   <sheetData>
     <row r="1" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A1" s="4" t="s">
-        <v>150</v>
+        <v>149</v>
       </c>
       <c r="B1" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="C1" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D1" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E1" s="5" t="s">
-        <v>252</v>
-      </c>
+        <v>133</v>
+      </c>
+      <c r="E1" s="5"/>
     </row>
     <row r="2" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A2" s="4" t="s">
-        <v>151</v>
+        <v>150</v>
       </c>
       <c r="B2" s="1" t="s">
-        <v>93</v>
+        <v>92</v>
       </c>
       <c r="C2" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D2" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E2" s="5" t="s">
-        <v>252</v>
-      </c>
+        <v>110</v>
+      </c>
+      <c r="E2" s="5"/>
     </row>
     <row r="3" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A3" s="4" t="s">
-        <v>172</v>
+        <v>171</v>
       </c>
       <c r="B3" s="1" t="s">
-        <v>81</v>
+        <v>80</v>
       </c>
       <c r="C3" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D3" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E3" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="4" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A4" s="4" t="s">
-        <v>177</v>
+        <v>176</v>
       </c>
       <c r="B4" s="1" t="s">
-        <v>82</v>
+        <v>81</v>
       </c>
       <c r="C4" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D4" s="3" t="s">
-        <v>119</v>
-      </c>
-      <c r="E4" t="s">
-        <v>252</v>
+        <v>118</v>
       </c>
     </row>
     <row r="5" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A5" s="4" t="s">
-        <v>155</v>
+        <v>154</v>
       </c>
       <c r="B5" s="1" t="s">
-        <v>100</v>
+        <v>99</v>
       </c>
       <c r="C5" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D5" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E5" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="6" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A6" s="4" t="s">
-        <v>236</v>
+        <v>235</v>
       </c>
       <c r="B6" s="1" t="s">
         <v>7</v>
       </c>
       <c r="C6" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D6" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E6" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="7" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A7" s="4" t="s">
-        <v>159</v>
+        <v>158</v>
       </c>
       <c r="B7" s="1" t="s">
-        <v>102</v>
+        <v>101</v>
       </c>
       <c r="C7" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D7" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E7" t="s">
-        <v>252</v>
+        <v>113</v>
       </c>
     </row>
     <row r="8" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A8" s="4" t="s">
-        <v>156</v>
+        <v>155</v>
       </c>
       <c r="B8" s="1" t="s">
-        <v>101</v>
+        <v>100</v>
       </c>
       <c r="C8" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="D8" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E8" t="s">
-        <v>252</v>
+        <v>110</v>
       </c>
     </row>
     <row r="9" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A9" s="4" t="s">
-        <v>158</v>
+        <v>157</v>
       </c>
       <c r="B9" s="1" t="s">
-        <v>106</v>
+        <v>105</v>
       </c>
       <c r="C9" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D9" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E9" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="10" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A10" s="4" t="s">
-        <v>198</v>
+        <v>197</v>
       </c>
       <c r="B10" s="1" t="s">
         <v>6</v>
       </c>
       <c r="C10" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D10" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E10" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="11" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A11" s="4" t="s">
-        <v>175</v>
+        <v>174</v>
       </c>
       <c r="B11" s="1" t="s">
         <v>8</v>
       </c>
       <c r="C11" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D11" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E11" t="s">
-        <v>252</v>
+        <v>113</v>
       </c>
     </row>
     <row r="12" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A12" s="4" t="s">
-        <v>174</v>
+        <v>173</v>
       </c>
       <c r="B12" s="1" t="s">
-        <v>84</v>
+        <v>83</v>
       </c>
       <c r="C12" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D12" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E12" t="s">
-        <v>252</v>
+        <v>112</v>
       </c>
     </row>
     <row r="13" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A13" s="4" t="s">
-        <v>196</v>
+        <v>195</v>
       </c>
       <c r="B13" s="1" t="s">
         <v>9</v>
       </c>
       <c r="C13" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D13" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E13" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="14" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A14" s="4" t="s">
-        <v>163</v>
+        <v>162</v>
       </c>
       <c r="B14" s="1" t="s">
-        <v>96</v>
+        <v>95</v>
       </c>
       <c r="C14" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D14" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E14" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="15" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A15" s="4" t="s">
-        <v>240</v>
+        <v>239</v>
       </c>
       <c r="B15" s="1" t="s">
         <v>10</v>
       </c>
       <c r="C15" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D15" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E15" t="s">
-        <v>252</v>
+        <v>113</v>
       </c>
     </row>
     <row r="16" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A16" s="4" t="s">
-        <v>206</v>
+        <v>205</v>
       </c>
       <c r="B16" s="1" t="s">
-        <v>74</v>
+        <v>73</v>
       </c>
       <c r="C16" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D16" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E16" t="s">
-        <v>252</v>
+        <v>111</v>
       </c>
     </row>
     <row r="17" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>239</v>
+        <v>238</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>11</v>
       </c>
       <c r="C17" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D17" s="3" t="s">
-        <v>113</v>
-      </c>
-      <c r="E17" t="s">
-        <v>252</v>
+        <v>112</v>
       </c>
     </row>
     <row r="18" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A18" s="4" t="s">
-        <v>167</v>
+        <v>166</v>
       </c>
       <c r="B18" s="1" t="s">
         <v>12</v>
       </c>
       <c r="C18" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>114</v>
-      </c>
-      <c r="E18" t="s">
-        <v>252</v>
+        <v>113</v>
       </c>
     </row>
     <row r="19" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>238</v>
+        <v>237</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="C19" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>112</v>
-      </c>
-      <c r="E19" t="s">
-        <v>252</v>
+        <v>111</v>
       </c>
     </row>
     <row r="20" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>171</v>
+        <v>170</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>260</v>
+        <v>258</v>
       </c>
       <c r="C20" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>118</v>
-      </c>
-      <c r="E20" t="s">
-        <v>252</v>
+        <v>117</v>
       </c>
     </row>
     <row r="21" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A21" s="4" t="s">
-        <v>189</v>
+        <v>188</v>
       </c>
       <c r="B21" s="1" t="s">
         <v>13</v>
       </c>
       <c r="C21" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E21" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="22" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>237</v>
+        <v>236</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="C22" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>111</v>
-      </c>
-      <c r="E22" t="s">
-        <v>252</v>
+        <v>110</v>
       </c>
     </row>
     <row r="23" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A23" s="4" t="s">
-        <v>166</v>
+        <v>165</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="C23" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>134</v>
-      </c>
-      <c r="E23" t="s">
-        <v>252</v>
+        <v>133</v>
       </c>
     </row>
     <row r="24" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A24" s="4" t="s">
-        <v>181</v>
+        <v>180</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>14</v>
       </c>
       <c r="C24" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D24" s="3" t="s">
-        <v>124</v>
-      </c>
-      <c r="E24" t="s">
-        <v>252</v>
+        <v>123</v>
       </c>
     </row>
     <row r="25" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>200</v>
+        <v>199</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>15</v>
       </c>
       <c r="C25" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D25" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="26" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>221</v>
+        <v>220</v>
       </c>
       <c r="B26" s="1" t="s">
-        <v>278</v>
+        <v>276</v>
       </c>
       <c r="C26" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D26" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
       <c r="F26" s="5"/>
     </row>
     <row r="27" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A27" s="4" t="s">
-        <v>153</v>
+        <v>152</v>
       </c>
       <c r="B27" s="1" t="s">
-        <v>94</v>
+        <v>93</v>
       </c>
       <c r="C27" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D27" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="E27" s="5"/>
     </row>
     <row r="28" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A28" s="4" t="s">
-        <v>169</v>
+        <v>168</v>
       </c>
       <c r="B28" s="1" t="s">
-        <v>257</v>
+        <v>255</v>
       </c>
       <c r="C28" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D28" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="29" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>232</v>
+        <v>231</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>16</v>
       </c>
       <c r="C29" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D29" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="30" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A30" s="4" t="s">
-        <v>170</v>
+        <v>169</v>
       </c>
       <c r="B30" s="1" t="s">
-        <v>258</v>
+        <v>256</v>
       </c>
       <c r="C30" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D30" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="31" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A31" s="4" t="s">
-        <v>202</v>
+        <v>201</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>17</v>
       </c>
       <c r="C31" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D31" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="32" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>231</v>
+        <v>230</v>
       </c>
       <c r="B32" s="1" t="s">
-        <v>290</v>
+        <v>288</v>
       </c>
       <c r="C32" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D32" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="33" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>210</v>
+        <v>209</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>20</v>
       </c>
       <c r="C33" s="3" t="s">
+        <v>117</v>
+      </c>
+      <c r="D33" s="3" t="s">
         <v>118</v>
-      </c>
-      <c r="D33" s="3" t="s">
-        <v>119</v>
       </c>
     </row>
     <row r="34" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A34" s="4" t="s">
-        <v>242</v>
+        <v>241</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>21</v>
       </c>
       <c r="C34" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D34" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="35" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A35" s="4" t="s">
-        <v>223</v>
+        <v>222</v>
       </c>
       <c r="B35" s="1" t="s">
-        <v>262</v>
+        <v>260</v>
       </c>
       <c r="C35" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D35" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
     </row>
     <row r="36" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A36" s="4" t="s">
-        <v>220</v>
+        <v>219</v>
       </c>
       <c r="B36" s="1" t="s">
-        <v>279</v>
+        <v>277</v>
       </c>
       <c r="C36" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D36" s="3" t="s">
-        <v>143</v>
+        <v>142</v>
       </c>
       <c r="F36" s="5"/>
     </row>
     <row r="37" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A37" s="4" t="s">
-        <v>203</v>
+        <v>202</v>
       </c>
       <c r="B37" s="1" t="s">
-        <v>275</v>
+        <v>273</v>
       </c>
       <c r="C37" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D37" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
       <c r="F37" s="5"/>
     </row>
     <row r="38" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A38" s="4" t="s">
-        <v>160</v>
+        <v>159</v>
       </c>
       <c r="B38" s="1" t="s">
-        <v>107</v>
+        <v>106</v>
       </c>
       <c r="C38" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D38" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="39" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A39" s="4" t="s">
-        <v>176</v>
+        <v>175</v>
       </c>
       <c r="B39" s="1" t="s">
-        <v>259</v>
+        <v>257</v>
       </c>
       <c r="C39" s="3" t="s">
+        <v>113</v>
+      </c>
+      <c r="D39" s="3" t="s">
         <v>114</v>
-      </c>
-      <c r="D39" s="3" t="s">
-        <v>115</v>
       </c>
     </row>
     <row r="40" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A40" s="4" t="s">
-        <v>165</v>
+        <v>164</v>
       </c>
       <c r="B40" s="1" t="s">
-        <v>288</v>
+        <v>286</v>
       </c>
       <c r="C40" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D40" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="F40" t="s">
-        <v>289</v>
+        <v>287</v>
       </c>
     </row>
     <row r="41" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A41" s="4" t="s">
-        <v>218</v>
+        <v>217</v>
       </c>
       <c r="B41" s="1" t="s">
-        <v>274</v>
+        <v>272</v>
       </c>
       <c r="C41" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D41" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
       <c r="F41" s="5"/>
     </row>
     <row r="42" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A42" s="4" t="s">
-        <v>207</v>
+        <v>206</v>
       </c>
       <c r="B42" s="1" t="s">
         <v>19</v>
       </c>
       <c r="C42" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D42" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="43" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A43" s="4" t="s">
-        <v>157</v>
+        <v>156</v>
       </c>
       <c r="B43" s="1" t="s">
+        <v>109</v>
+      </c>
+      <c r="C43" s="3" t="s">
         <v>110</v>
       </c>
-      <c r="C43" s="3" t="s">
+      <c r="D43" s="3" t="s">
         <v>111</v>
-      </c>
-      <c r="D43" s="3" t="s">
-        <v>112</v>
       </c>
     </row>
     <row r="44" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A44" s="4" t="s">
-        <v>204</v>
+        <v>203</v>
       </c>
       <c r="B44" s="1" t="s">
         <v>22</v>
       </c>
       <c r="C44" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D44" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="45" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A45" s="4" t="s">
-        <v>197</v>
+        <v>196</v>
       </c>
       <c r="B45" s="1" t="s">
-        <v>271</v>
+        <v>269</v>
       </c>
       <c r="C45" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D45" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
+      </c>
+      <c r="F45" t="s">
+        <v>313</v>
       </c>
     </row>
     <row r="46" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A46" s="4" t="s">
-        <v>208</v>
+        <v>207</v>
       </c>
       <c r="B46" s="1" t="s">
         <v>23</v>
       </c>
       <c r="C46" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D46" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="47" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A47" s="4" t="s">
-        <v>247</v>
+        <v>246</v>
       </c>
       <c r="B47" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="C47" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D47" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="48" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A48" s="4" t="s">
-        <v>154</v>
+        <v>153</v>
       </c>
       <c r="B48" s="1" t="s">
-        <v>95</v>
+        <v>94</v>
       </c>
       <c r="C48" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D48" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="49" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A49" s="4" t="s">
-        <v>244</v>
+        <v>243</v>
       </c>
       <c r="B49" s="1" t="s">
-        <v>277</v>
+        <v>275</v>
       </c>
       <c r="C49" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D49" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
       <c r="F49" s="5"/>
     </row>
     <row r="50" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A50" s="4" t="s">
-        <v>226</v>
+        <v>225</v>
       </c>
       <c r="B50" s="1" t="s">
         <v>25</v>
       </c>
       <c r="C50" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D50" s="3" t="s">
-        <v>148</v>
+        <v>147</v>
       </c>
     </row>
     <row r="51" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A51" s="4" t="s">
-        <v>180</v>
+        <v>179</v>
       </c>
       <c r="B51" s="1" t="s">
         <v>26</v>
       </c>
       <c r="C51" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D51" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="52" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A52" s="4" t="s">
-        <v>183</v>
+        <v>182</v>
       </c>
       <c r="B52" s="1" t="s">
         <v>27</v>
       </c>
       <c r="C52" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D52" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="53" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A53" s="4" t="s">
-        <v>179</v>
+        <v>178</v>
       </c>
       <c r="B53" s="1" t="s">
         <v>28</v>
       </c>
       <c r="C53" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D53" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="54" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A54" s="4" t="s">
-        <v>205</v>
+        <v>204</v>
       </c>
       <c r="B54" s="1" t="s">
         <v>29</v>
       </c>
       <c r="C54" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D54" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="55" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A55" s="4" t="s">
-        <v>199</v>
+        <v>198</v>
       </c>
       <c r="B55" s="1" t="s">
         <v>30</v>
       </c>
       <c r="C55" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D55" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="56" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A56" s="4" t="s">
-        <v>190</v>
+        <v>189</v>
       </c>
       <c r="B56" s="1" t="s">
         <v>31</v>
       </c>
       <c r="C56" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D56" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="57" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A57" s="4" t="s">
-        <v>191</v>
+        <v>190</v>
       </c>
       <c r="B57" s="1" t="s">
         <v>32</v>
       </c>
       <c r="C57" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D57" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="58" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A58" s="4" t="s">
-        <v>173</v>
+        <v>172</v>
       </c>
       <c r="B58" s="1" t="s">
         <v>33</v>
       </c>
       <c r="C58" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D58" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="59" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A59" s="4" t="s">
-        <v>222</v>
+        <v>221</v>
       </c>
       <c r="B59" s="1" t="s">
         <v>24</v>
       </c>
       <c r="C59" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D59" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="60" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A60" s="4" t="s">
-        <v>211</v>
+        <v>210</v>
       </c>
       <c r="B60" s="1" t="s">
         <v>34</v>
       </c>
       <c r="C60" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D60" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="61" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A61" s="4" t="s">
-        <v>217</v>
+        <v>216</v>
       </c>
       <c r="B61" s="1" t="s">
-        <v>276</v>
+        <v>274</v>
       </c>
       <c r="C61" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D61" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
       <c r="F61" s="5"/>
     </row>
     <row r="62" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A62" s="4" t="s">
-        <v>152</v>
+        <v>151</v>
       </c>
       <c r="B62" s="1" t="s">
-        <v>251</v>
+        <v>250</v>
       </c>
       <c r="C62" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D62" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="E62" s="5"/>
     </row>
     <row r="63" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A63" s="4" t="s">
-        <v>214</v>
+        <v>213</v>
       </c>
       <c r="B63" s="1" t="s">
         <v>40</v>
       </c>
       <c r="C63" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D63" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="64" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A64" s="4" t="s">
-        <v>209</v>
+        <v>208</v>
       </c>
       <c r="B64" s="1" t="s">
         <v>41</v>
       </c>
       <c r="C64" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D64" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="65" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A65" s="4" t="s">
-        <v>212</v>
+        <v>211</v>
       </c>
       <c r="B65" s="1" t="s">
         <v>42</v>
       </c>
       <c r="C65" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D65" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="66" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A66" s="4" t="s">
-        <v>161</v>
+        <v>160</v>
       </c>
       <c r="B66" s="1" t="s">
-        <v>105</v>
+        <v>104</v>
       </c>
       <c r="C66" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D66" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="67" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A67" s="4" t="s">
-        <v>248</v>
+        <v>247</v>
       </c>
       <c r="B67" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="C67" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D67" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="68" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A68" s="4" t="s">
-        <v>245</v>
+        <v>244</v>
       </c>
       <c r="B68" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="C68" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
       <c r="D68" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="69" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A69" s="4" t="s">
-        <v>168</v>
+        <v>167</v>
       </c>
       <c r="B69" s="1" t="s">
-        <v>254</v>
+        <v>252</v>
       </c>
       <c r="C69" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D69" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="70" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A70" s="4" t="s">
-        <v>162</v>
+        <v>161</v>
       </c>
       <c r="B70" s="1" t="s">
-        <v>109</v>
+        <v>108</v>
       </c>
       <c r="C70" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D70" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="71" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A71" s="4" t="s">
-        <v>225</v>
+        <v>224</v>
       </c>
       <c r="B71" s="1" t="s">
         <v>43</v>
       </c>
       <c r="C71" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D71" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="72" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A72" s="4" t="s">
-        <v>227</v>
+        <v>226</v>
       </c>
       <c r="B72" s="1" t="s">
         <v>44</v>
       </c>
       <c r="C72" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D72" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="73" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A73" s="4" t="s">
-        <v>228</v>
+        <v>227</v>
       </c>
       <c r="B73" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="C73" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D73" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="74" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A74" s="4" t="s">
-        <v>193</v>
+        <v>192</v>
       </c>
       <c r="B74" s="1" t="s">
         <v>45</v>
       </c>
       <c r="C74" s="3" t="s">
+        <v>114</v>
+      </c>
+      <c r="D74" s="3" t="s">
         <v>115</v>
-      </c>
-      <c r="D74" s="3" t="s">
-        <v>116</v>
       </c>
     </row>
     <row r="75" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A75" s="4" t="s">
-        <v>246</v>
+        <v>245</v>
       </c>
       <c r="B75" s="1" t="s">
-        <v>98</v>
+        <v>97</v>
       </c>
       <c r="C75" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D75" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="76" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A76" s="4" t="s">
-        <v>215</v>
+        <v>214</v>
       </c>
       <c r="B76" s="1" t="s">
         <v>46</v>
       </c>
       <c r="C76" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D76" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="77" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A77" s="4" t="s">
-        <v>194</v>
+        <v>193</v>
       </c>
       <c r="B77" s="1" t="s">
-        <v>267</v>
+        <v>265</v>
       </c>
       <c r="C77" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D77" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="78" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A78" s="4" t="s">
-        <v>201</v>
+        <v>200</v>
       </c>
       <c r="B78" s="1" t="s">
         <v>47</v>
       </c>
       <c r="C78" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D78" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="79" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A79" s="4" t="s">
-        <v>241</v>
+        <v>240</v>
       </c>
       <c r="B79" s="1" t="s">
         <v>48</v>
       </c>
       <c r="C79" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D79" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="80" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A80" s="4" t="s">
-        <v>219</v>
+        <v>218</v>
       </c>
       <c r="B80" s="1" t="s">
-        <v>273</v>
+        <v>271</v>
       </c>
       <c r="C80" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D80" s="3" t="s">
-        <v>144</v>
+        <v>143</v>
       </c>
       <c r="F80" s="5"/>
     </row>
     <row r="81" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A81" s="4" t="s">
-        <v>229</v>
+        <v>228</v>
       </c>
       <c r="B81" s="1" t="s">
         <v>0</v>
       </c>
       <c r="C81" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D81" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="82" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A82" s="4" t="s">
-        <v>243</v>
+        <v>242</v>
       </c>
       <c r="B82" s="1" t="s">
         <v>49</v>
       </c>
       <c r="C82" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D82" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="83" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A83" s="4" t="s">
-        <v>195</v>
+        <v>194</v>
       </c>
       <c r="B83" s="1" t="s">
         <v>50</v>
       </c>
       <c r="C83" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D83" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="84" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A84" s="4" t="s">
-        <v>233</v>
+        <v>232</v>
       </c>
       <c r="B84" s="1" t="s">
         <v>51</v>
       </c>
       <c r="C84" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D84" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="85" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A85" s="4" t="s">
-        <v>230</v>
+        <v>229</v>
       </c>
       <c r="B85" s="1" t="s">
         <v>52</v>
       </c>
       <c r="C85" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D85" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="86" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A86" s="4" t="s">
-        <v>234</v>
+        <v>233</v>
       </c>
       <c r="B86" s="1" t="s">
-        <v>295</v>
+        <v>293</v>
       </c>
       <c r="C86" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D86" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="87" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A87" s="4" t="s">
-        <v>216</v>
+        <v>215</v>
       </c>
       <c r="B87" s="1" t="s">
-        <v>75</v>
+        <v>74</v>
       </c>
       <c r="C87" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D87" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="88" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A88" s="4" t="s">
-        <v>164</v>
+        <v>163</v>
       </c>
       <c r="B88" s="1" t="s">
-        <v>97</v>
+        <v>96</v>
       </c>
       <c r="C88" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D88" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="89" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A89" s="4" t="s">
-        <v>182</v>
+        <v>181</v>
       </c>
       <c r="B89" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="C89" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D89" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="90" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A90" s="4" t="s">
-        <v>213</v>
+        <v>212</v>
       </c>
       <c r="B90" s="1" t="s">
-        <v>80</v>
+        <v>79</v>
       </c>
       <c r="C90" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D90" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="91" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A91" s="4" t="s">
-        <v>178</v>
+        <v>177</v>
       </c>
       <c r="B91" s="1" t="s">
         <v>53</v>
       </c>
       <c r="C91" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D91" s="3" t="s">
-        <v>132</v>
+        <v>131</v>
       </c>
     </row>
     <row r="92" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A92" s="4" t="s">
-        <v>185</v>
+        <v>184</v>
       </c>
       <c r="B92" s="1" t="s">
         <v>54</v>
       </c>
       <c r="C92" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D92" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="93" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A93" s="4" t="s">
-        <v>186</v>
+        <v>185</v>
       </c>
       <c r="B93" s="1" t="s">
         <v>55</v>
       </c>
       <c r="C93" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D93" s="3" t="s">
-        <v>139</v>
+        <v>138</v>
       </c>
     </row>
     <row r="94" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A94" s="4" t="s">
-        <v>187</v>
+        <v>186</v>
       </c>
       <c r="B94" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="C94" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D94" s="3" t="s">
-        <v>140</v>
+        <v>139</v>
       </c>
     </row>
     <row r="95" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A95" s="4" t="s">
-        <v>235</v>
+        <v>234</v>
       </c>
       <c r="B95" s="1" t="s">
         <v>1</v>
       </c>
       <c r="C95" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D95" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="96" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A96" s="4" t="s">
-        <v>192</v>
+        <v>191</v>
       </c>
       <c r="B96" s="1" t="s">
-        <v>266</v>
+        <v>264</v>
       </c>
       <c r="C96" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D96" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="97" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A97" s="4" t="s">
-        <v>224</v>
+        <v>223</v>
       </c>
       <c r="B97" s="1" t="s">
-        <v>294</v>
+        <v>292</v>
       </c>
       <c r="C97" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D97" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="98" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A98" s="4" t="s">
-        <v>184</v>
+        <v>183</v>
       </c>
       <c r="B98" s="1" t="s">
-        <v>85</v>
+        <v>84</v>
       </c>
       <c r="C98" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D98" s="3" t="s">
-        <v>126</v>
+        <v>125</v>
       </c>
     </row>
     <row r="99" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A99" s="4" t="s">
-        <v>188</v>
+        <v>187</v>
       </c>
       <c r="B99" s="1" t="s">
         <v>56</v>
       </c>
       <c r="C99" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D99" s="3" t="s">
-        <v>141</v>
+        <v>140</v>
       </c>
     </row>
     <row r="100" spans="1:6" x14ac:dyDescent="0.3">
@@ -2884,10 +2817,10 @@
         <v>57</v>
       </c>
       <c r="C100" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D100" s="3" t="s">
-        <v>142</v>
+        <v>141</v>
       </c>
     </row>
     <row r="101" spans="1:6" x14ac:dyDescent="0.3">
@@ -2895,13 +2828,13 @@
         <v>101</v>
       </c>
       <c r="B101" s="1" t="s">
-        <v>261</v>
+        <v>259</v>
       </c>
       <c r="C101" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D101" s="3" t="s">
-        <v>137</v>
+        <v>136</v>
       </c>
     </row>
     <row r="102" spans="1:6" x14ac:dyDescent="0.3">
@@ -2912,24 +2845,24 @@
         <v>58</v>
       </c>
       <c r="C102" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D102" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="103" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A103" s="4" t="s">
-        <v>280</v>
+        <v>278</v>
       </c>
       <c r="B103" s="1" t="s">
-        <v>284</v>
+        <v>282</v>
       </c>
       <c r="C103" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D103" s="3" t="s">
-        <v>146</v>
+        <v>145</v>
       </c>
     </row>
     <row r="104" spans="1:6" x14ac:dyDescent="0.3">
@@ -2937,13 +2870,13 @@
         <v>104</v>
       </c>
       <c r="B104" s="1" t="s">
-        <v>79</v>
+        <v>78</v>
       </c>
       <c r="C104" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D104" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="105" spans="1:6" x14ac:dyDescent="0.3">
@@ -2951,13 +2884,13 @@
         <v>105</v>
       </c>
       <c r="B105" s="1" t="s">
-        <v>250</v>
+        <v>249</v>
       </c>
       <c r="C105" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D105" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="E105" s="5"/>
     </row>
@@ -2969,10 +2902,10 @@
         <v>35</v>
       </c>
       <c r="C106" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D106" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="107" spans="1:6" x14ac:dyDescent="0.3">
@@ -2980,13 +2913,13 @@
         <v>107</v>
       </c>
       <c r="B107" s="1" t="s">
-        <v>269</v>
+        <v>267</v>
       </c>
       <c r="C107" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D107" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="108" spans="1:6" x14ac:dyDescent="0.3">
@@ -2994,13 +2927,13 @@
         <v>108</v>
       </c>
       <c r="B108" s="1" t="s">
-        <v>78</v>
+        <v>77</v>
       </c>
       <c r="C108" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D108" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="109" spans="1:6" x14ac:dyDescent="0.3">
@@ -3011,10 +2944,10 @@
         <v>2</v>
       </c>
       <c r="C109" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D109" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="110" spans="1:6" x14ac:dyDescent="0.3">
@@ -3025,27 +2958,27 @@
         <v>36</v>
       </c>
       <c r="C110" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D110" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="111" spans="1:6" x14ac:dyDescent="0.3">
       <c r="A111" s="4" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="B111" s="1" t="s">
-        <v>135</v>
+        <v>134</v>
       </c>
       <c r="C111" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D111" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
       <c r="F111" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
     </row>
     <row r="112" spans="1:6" x14ac:dyDescent="0.3">
@@ -3056,10 +2989,10 @@
         <v>3</v>
       </c>
       <c r="C112" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D112" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="113" spans="1:4" x14ac:dyDescent="0.3">
@@ -3070,10 +3003,10 @@
         <v>37</v>
       </c>
       <c r="C113" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D113" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="114" spans="1:4" x14ac:dyDescent="0.3">
@@ -3084,10 +3017,10 @@
         <v>38</v>
       </c>
       <c r="C114" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D114" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="115" spans="1:4" x14ac:dyDescent="0.3">
@@ -3095,13 +3028,13 @@
         <v>115</v>
       </c>
       <c r="B115" s="1" t="s">
-        <v>77</v>
+        <v>76</v>
       </c>
       <c r="C115" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D115" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="116" spans="1:4" x14ac:dyDescent="0.3">
@@ -3109,13 +3042,13 @@
         <v>116</v>
       </c>
       <c r="B116" s="1" t="s">
-        <v>104</v>
+        <v>103</v>
       </c>
       <c r="C116" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D116" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="117" spans="1:4" x14ac:dyDescent="0.3">
@@ -3123,13 +3056,13 @@
         <v>117</v>
       </c>
       <c r="B117" s="1" t="s">
-        <v>255</v>
+        <v>253</v>
       </c>
       <c r="C117" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D117" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="118" spans="1:4" x14ac:dyDescent="0.3">
@@ -3137,13 +3070,13 @@
         <v>118</v>
       </c>
       <c r="B118" s="1" t="s">
-        <v>283</v>
+        <v>281</v>
       </c>
       <c r="C118" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D118" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="119" spans="1:4" x14ac:dyDescent="0.3">
@@ -3151,13 +3084,13 @@
         <v>119</v>
       </c>
       <c r="B119" s="1" t="s">
-        <v>282</v>
+        <v>280</v>
       </c>
       <c r="C119" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D119" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
     </row>
     <row r="120" spans="1:4" x14ac:dyDescent="0.3">
@@ -3165,13 +3098,13 @@
         <v>120</v>
       </c>
       <c r="B120" s="1" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="C120" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
       <c r="D120" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="121" spans="1:4" x14ac:dyDescent="0.3">
@@ -3179,13 +3112,13 @@
         <v>121</v>
       </c>
       <c r="B121" s="1" t="s">
-        <v>287</v>
+        <v>285</v>
       </c>
       <c r="C121" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D121" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="122" spans="1:4" x14ac:dyDescent="0.3">
@@ -3193,13 +3126,13 @@
         <v>122</v>
       </c>
       <c r="B122" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="C122" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D122" s="3" t="s">
-        <v>122</v>
+        <v>121</v>
       </c>
     </row>
     <row r="123" spans="1:4" x14ac:dyDescent="0.3">
@@ -3210,10 +3143,10 @@
         <v>39</v>
       </c>
       <c r="C123" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D123" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="124" spans="1:4" x14ac:dyDescent="0.3">
@@ -3221,13 +3154,13 @@
         <v>124</v>
       </c>
       <c r="B124" s="1" t="s">
-        <v>103</v>
+        <v>102</v>
       </c>
       <c r="C124" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="D124" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="125" spans="1:4" x14ac:dyDescent="0.3">
@@ -3235,13 +3168,13 @@
         <v>125</v>
       </c>
       <c r="B125" s="1" t="s">
-        <v>136</v>
+        <v>135</v>
       </c>
       <c r="C125" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
       <c r="D125" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
     <row r="126" spans="1:4" x14ac:dyDescent="0.3">
@@ -3252,10 +3185,10 @@
         <v>59</v>
       </c>
       <c r="C126" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D126" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="127" spans="1:4" x14ac:dyDescent="0.3">
@@ -3263,13 +3196,13 @@
         <v>127</v>
       </c>
       <c r="B127" s="1" t="s">
-        <v>89</v>
+        <v>88</v>
       </c>
       <c r="C127" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D127" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="128" spans="1:4" x14ac:dyDescent="0.3">
@@ -3277,13 +3210,13 @@
         <v>128</v>
       </c>
       <c r="B128" s="1" t="s">
-        <v>108</v>
+        <v>107</v>
       </c>
       <c r="C128" s="3" t="s">
+        <v>111</v>
+      </c>
+      <c r="D128" s="3" t="s">
         <v>112</v>
-      </c>
-      <c r="D128" s="3" t="s">
-        <v>113</v>
       </c>
     </row>
     <row r="129" spans="1:5" x14ac:dyDescent="0.3">
@@ -3291,13 +3224,13 @@
         <v>129</v>
       </c>
       <c r="B129" s="1" t="s">
-        <v>90</v>
+        <v>89</v>
       </c>
       <c r="C129" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D129" s="3" t="s">
-        <v>111</v>
+        <v>110</v>
       </c>
     </row>
     <row r="130" spans="1:5" x14ac:dyDescent="0.3">
@@ -3308,10 +3241,10 @@
         <v>60</v>
       </c>
       <c r="C130" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D130" s="3" t="s">
-        <v>133</v>
+        <v>132</v>
       </c>
     </row>
     <row r="131" spans="1:5" x14ac:dyDescent="0.3">
@@ -3319,13 +3252,13 @@
         <v>131</v>
       </c>
       <c r="B131" s="1" t="s">
-        <v>286</v>
+        <v>284</v>
       </c>
       <c r="C131" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D131" s="3" t="s">
-        <v>145</v>
+        <v>144</v>
       </c>
     </row>
     <row r="132" spans="1:5" x14ac:dyDescent="0.3">
@@ -3333,13 +3266,13 @@
         <v>132</v>
       </c>
       <c r="B132" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="C132" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D132" s="3" t="s">
-        <v>123</v>
+        <v>122</v>
       </c>
     </row>
     <row r="133" spans="1:5" x14ac:dyDescent="0.3">
@@ -3347,13 +3280,13 @@
         <v>133</v>
       </c>
       <c r="B133" s="1" t="s">
-        <v>293</v>
+        <v>291</v>
       </c>
       <c r="C133" s="3" t="s">
+        <v>120</v>
+      </c>
+      <c r="D133" s="3" t="s">
         <v>121</v>
-      </c>
-      <c r="D133" s="3" t="s">
-        <v>122</v>
       </c>
     </row>
     <row r="134" spans="1:5" x14ac:dyDescent="0.3">
@@ -3361,13 +3294,13 @@
         <v>134</v>
       </c>
       <c r="B134" s="1" t="s">
-        <v>87</v>
+        <v>86</v>
       </c>
       <c r="C134" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D134" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="135" spans="1:5" x14ac:dyDescent="0.3">
@@ -3375,13 +3308,13 @@
         <v>135</v>
       </c>
       <c r="B135" s="1" t="s">
-        <v>292</v>
+        <v>290</v>
       </c>
       <c r="C135" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D135" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="136" spans="1:5" x14ac:dyDescent="0.3">
@@ -3389,13 +3322,13 @@
         <v>136</v>
       </c>
       <c r="B136" s="1" t="s">
-        <v>272</v>
+        <v>270</v>
       </c>
       <c r="C136" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D136" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="137" spans="1:5" x14ac:dyDescent="0.3">
@@ -3403,13 +3336,13 @@
         <v>137</v>
       </c>
       <c r="B137" s="1" t="s">
-        <v>253</v>
+        <v>251</v>
       </c>
       <c r="C137" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D137" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="138" spans="1:5" x14ac:dyDescent="0.3">
@@ -3417,13 +3350,13 @@
         <v>138</v>
       </c>
       <c r="B138" s="1" t="s">
-        <v>62</v>
+        <v>315</v>
       </c>
       <c r="C138" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D138" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="139" spans="1:5" x14ac:dyDescent="0.3">
@@ -3431,13 +3364,13 @@
         <v>139</v>
       </c>
       <c r="B139" s="1" t="s">
-        <v>63</v>
+        <v>62</v>
       </c>
       <c r="C139" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D139" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="140" spans="1:5" x14ac:dyDescent="0.3">
@@ -3445,13 +3378,13 @@
         <v>140</v>
       </c>
       <c r="B140" s="1" t="s">
-        <v>64</v>
+        <v>63</v>
       </c>
       <c r="C140" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D140" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="141" spans="1:5" x14ac:dyDescent="0.3">
@@ -3459,13 +3392,13 @@
         <v>141</v>
       </c>
       <c r="B141" s="1" t="s">
-        <v>86</v>
+        <v>85</v>
       </c>
       <c r="C141" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D141" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="142" spans="1:5" x14ac:dyDescent="0.3">
@@ -3476,24 +3409,24 @@
         <v>61</v>
       </c>
       <c r="C142" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D142" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
     </row>
     <row r="143" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A143" s="4" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="B143" s="1" t="s">
-        <v>270</v>
+        <v>268</v>
       </c>
       <c r="C143" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D143" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="144" spans="1:5" x14ac:dyDescent="0.3">
@@ -3501,13 +3434,13 @@
         <v>144</v>
       </c>
       <c r="B144" s="1" t="s">
-        <v>92</v>
+        <v>91</v>
       </c>
       <c r="C144" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D144" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
       <c r="E144" s="5"/>
     </row>
@@ -3516,13 +3449,13 @@
         <v>145</v>
       </c>
       <c r="B145" s="1" t="s">
-        <v>65</v>
+        <v>64</v>
       </c>
       <c r="C145" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D145" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="146" spans="1:4" x14ac:dyDescent="0.3">
@@ -3530,13 +3463,13 @@
         <v>146</v>
       </c>
       <c r="B146" s="1" t="s">
-        <v>66</v>
+        <v>65</v>
       </c>
       <c r="C146" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D146" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="147" spans="1:4" x14ac:dyDescent="0.3">
@@ -3544,13 +3477,13 @@
         <v>147</v>
       </c>
       <c r="B147" s="1" t="s">
-        <v>256</v>
+        <v>254</v>
       </c>
       <c r="C147" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D147" s="3" t="s">
-        <v>119</v>
+        <v>118</v>
       </c>
     </row>
     <row r="148" spans="1:4" x14ac:dyDescent="0.3">
@@ -3558,13 +3491,13 @@
         <v>148</v>
       </c>
       <c r="B148" s="1" t="s">
-        <v>285</v>
+        <v>283</v>
       </c>
       <c r="C148" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D148" s="3" t="s">
-        <v>147</v>
+        <v>146</v>
       </c>
     </row>
     <row r="149" spans="1:4" x14ac:dyDescent="0.3">
@@ -3575,10 +3508,10 @@
         <v>4</v>
       </c>
       <c r="C149" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D149" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
     </row>
     <row r="150" spans="1:4" x14ac:dyDescent="0.3">
@@ -3586,13 +3519,13 @@
         <v>150</v>
       </c>
       <c r="B150" s="1" t="s">
-        <v>296</v>
+        <v>294</v>
       </c>
       <c r="C150" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D150" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="151" spans="1:4" x14ac:dyDescent="0.3">
@@ -3600,13 +3533,13 @@
         <v>151</v>
       </c>
       <c r="B151" s="1" t="s">
-        <v>88</v>
+        <v>87</v>
       </c>
       <c r="C151" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
       <c r="D151" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
     </row>
     <row r="152" spans="1:4" x14ac:dyDescent="0.3">
@@ -3614,13 +3547,13 @@
         <v>152</v>
       </c>
       <c r="B152" s="1" t="s">
-        <v>297</v>
+        <v>314</v>
       </c>
       <c r="C152" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D152" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="153" spans="1:4" x14ac:dyDescent="0.3">
@@ -3628,13 +3561,13 @@
         <v>153</v>
       </c>
       <c r="B153" s="1" t="s">
-        <v>67</v>
+        <v>66</v>
       </c>
       <c r="C153" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D153" s="3" t="s">
-        <v>127</v>
+        <v>126</v>
       </c>
     </row>
     <row r="154" spans="1:4" x14ac:dyDescent="0.3">
@@ -3642,13 +3575,13 @@
         <v>154</v>
       </c>
       <c r="B154" s="1" t="s">
-        <v>83</v>
+        <v>82</v>
       </c>
       <c r="C154" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D154" s="3" t="s">
-        <v>131</v>
+        <v>130</v>
       </c>
     </row>
     <row r="155" spans="1:4" x14ac:dyDescent="0.3">
@@ -3656,13 +3589,13 @@
         <v>155</v>
       </c>
       <c r="B155" s="1" t="s">
-        <v>68</v>
+        <v>67</v>
       </c>
       <c r="C155" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D155" s="3" t="s">
-        <v>129</v>
+        <v>128</v>
       </c>
     </row>
     <row r="156" spans="1:4" x14ac:dyDescent="0.3">
@@ -3670,13 +3603,13 @@
         <v>156</v>
       </c>
       <c r="B156" s="1" t="s">
-        <v>291</v>
+        <v>289</v>
       </c>
       <c r="C156" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D156" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="157" spans="1:4" x14ac:dyDescent="0.3">
@@ -3684,13 +3617,13 @@
         <v>157</v>
       </c>
       <c r="B157" s="1" t="s">
-        <v>69</v>
+        <v>68</v>
       </c>
       <c r="C157" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D157" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="158" spans="1:4" x14ac:dyDescent="0.3">
@@ -3698,13 +3631,13 @@
         <v>158</v>
       </c>
       <c r="B158" s="1" t="s">
-        <v>70</v>
+        <v>69</v>
       </c>
       <c r="C158" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D158" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="159" spans="1:4" x14ac:dyDescent="0.3">
@@ -3712,13 +3645,13 @@
         <v>159</v>
       </c>
       <c r="B159" s="1" t="s">
-        <v>76</v>
+        <v>75</v>
       </c>
       <c r="C159" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D159" s="3" t="s">
-        <v>149</v>
+        <v>148</v>
       </c>
     </row>
     <row r="160" spans="1:4" x14ac:dyDescent="0.3">
@@ -3726,13 +3659,13 @@
         <v>160</v>
       </c>
       <c r="B160" s="1" t="s">
-        <v>281</v>
+        <v>279</v>
       </c>
       <c r="C160" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
       <c r="D160" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
     </row>
     <row r="161" spans="1:4" x14ac:dyDescent="0.3">
@@ -3743,52 +3676,52 @@
         <v>5</v>
       </c>
       <c r="C161" s="3" t="s">
-        <v>120</v>
+        <v>119</v>
       </c>
       <c r="D161" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
     </row>
     <row r="162" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A162" s="4" t="s">
-        <v>263</v>
+        <v>261</v>
       </c>
       <c r="B162" s="1" t="s">
         <v>18</v>
       </c>
       <c r="C162" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
       <c r="D162" s="3" t="s">
-        <v>115</v>
+        <v>114</v>
       </c>
     </row>
     <row r="163" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A163" s="4" t="s">
-        <v>264</v>
+        <v>262</v>
       </c>
       <c r="B163" s="1" t="s">
-        <v>265</v>
+        <v>263</v>
       </c>
       <c r="C163" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D163" s="3" t="s">
-        <v>138</v>
+        <v>137</v>
       </c>
     </row>
     <row r="164" spans="1:4" x14ac:dyDescent="0.3">
       <c r="A164" s="4" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="B164" s="1" t="s">
-        <v>268</v>
+        <v>266</v>
       </c>
       <c r="C164" s="3" t="s">
-        <v>116</v>
+        <v>115</v>
       </c>
       <c r="D164" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="165" spans="1:4" x14ac:dyDescent="0.3">
@@ -3796,13 +3729,13 @@
         <v>165</v>
       </c>
       <c r="B165" s="1" t="s">
-        <v>91</v>
+        <v>90</v>
       </c>
       <c r="C165" s="3" t="s">
-        <v>113</v>
+        <v>112</v>
       </c>
       <c r="D165" s="3" t="s">
-        <v>112</v>
+        <v>111</v>
       </c>
     </row>
     <row r="166" spans="1:4" x14ac:dyDescent="0.3">
@@ -3810,13 +3743,13 @@
         <v>166</v>
       </c>
       <c r="B166" s="1" t="s">
-        <v>99</v>
+        <v>98</v>
       </c>
       <c r="C166" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
       <c r="D166" s="3" t="s">
-        <v>117</v>
+        <v>116</v>
       </c>
     </row>
     <row r="167" spans="1:4" x14ac:dyDescent="0.3">
@@ -3824,13 +3757,13 @@
         <v>167</v>
       </c>
       <c r="B167" s="1" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="C167" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D167" s="3" t="s">
-        <v>128</v>
+        <v>127</v>
       </c>
     </row>
     <row r="168" spans="1:4" x14ac:dyDescent="0.3">
@@ -3838,13 +3771,13 @@
         <v>168</v>
       </c>
       <c r="B168" s="1" t="s">
-        <v>73</v>
+        <v>72</v>
       </c>
       <c r="C168" s="3" t="s">
-        <v>118</v>
+        <v>117</v>
       </c>
       <c r="D168" s="3" t="s">
-        <v>121</v>
+        <v>120</v>
       </c>
     </row>
     <row r="169" spans="1:4" x14ac:dyDescent="0.3">
@@ -3852,13 +3785,13 @@
         <v>169</v>
       </c>
       <c r="B169" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="C169" s="3" t="s">
-        <v>124</v>
+        <v>123</v>
       </c>
       <c r="D169" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
     </row>
     <row r="170" spans="1:4" x14ac:dyDescent="0.3">
@@ -3866,13 +3799,13 @@
         <v>170</v>
       </c>
       <c r="B170" s="1" t="s">
-        <v>72</v>
+        <v>71</v>
       </c>
       <c r="C170" s="3" t="s">
-        <v>114</v>
+        <v>113</v>
       </c>
       <c r="D170" s="3" t="s">
-        <v>130</v>
+        <v>129</v>
       </c>
     </row>
     <row r="171" spans="1:4" x14ac:dyDescent="0.3">
@@ -3880,13 +3813,13 @@
         <v>171</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>249</v>
+        <v>248</v>
       </c>
       <c r="C171" s="3" t="s">
-        <v>125</v>
+        <v>124</v>
       </c>
       <c r="D171" s="3" t="s">
-        <v>134</v>
+        <v>133</v>
       </c>
     </row>
   </sheetData>

</xml_diff>

<commit_message>
added some proverb images
</commit_message>
<xml_diff>
--- a/p/content_by_grammar.xlsx
+++ b/p/content_by_grammar.xlsx
@@ -8,7 +8,7 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="C:\Users\adsv\private\books\language\ingush\Dahkilgov\github\dahkilgov\p\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{C3B66E2D-69F3-47E7-8590-67B3ADC6F1D2}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{7DCD93DD-3EAA-4BB2-8730-85D65C5E06ED}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
     <workbookView xWindow="28680" yWindow="-2415" windowWidth="38640" windowHeight="21120" xr2:uid="{AC639D1C-64A7-45F6-9CFA-A1A688E9895B}"/>
   </bookViews>
@@ -16,7 +16,6 @@
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
   </sheets>
   <calcPr calcId="191029"/>
-  <fileRecoveryPr repairLoad="1"/>
   <extLst>
     <ext xmlns:x15="http://schemas.microsoft.com/office/spreadsheetml/2010/11/main" uri="{140A7094-0E35-4892-8432-C4D2E57EDEB5}">
       <x15:workbookPr chartTrackingRefBase="1"/>
@@ -576,9 +575,6 @@
     <t>Составные слова, фразеологические обороты.</t>
   </si>
   <si>
-    <t>Пространственные послелоги тIа, чу, ...</t>
-  </si>
-  <si>
     <t>Составные послелоги, гӀолла.</t>
   </si>
   <si>
@@ -594,9 +590,6 @@
     <t>Частицы -о, -а для обозначения долготы действия.</t>
   </si>
   <si>
-    <t>Вопросительное предложение. Общие сведения.</t>
-  </si>
-  <si>
     <t>Вопросительное предложение, слово «фуд».</t>
   </si>
   <si>
@@ -729,9 +722,6 @@
     <t>Суффиксы для абстрактных понятий.</t>
   </si>
   <si>
-    <t>Отглагольное существительное с суффиксом "лга".</t>
-  </si>
-  <si>
     <t>Падежи, общие сведения.</t>
   </si>
   <si>
@@ -999,7 +989,16 @@
     <t>Грамматика</t>
   </si>
   <si>
-    <t>Пространственная приставка «ура-», вертикальный.</t>
+    <t>Пространственные послелоги, использование с существительными.</t>
+  </si>
+  <si>
+    <t>Пространственные послелоги, использование с глаголами.</t>
+  </si>
+  <si>
+    <t>Конструкция вопросительного предложения.</t>
+  </si>
+  <si>
+    <t>Суффиксы для отглагольных существительных.</t>
   </si>
 </sst>
 </file>
@@ -1446,7 +1445,7 @@
         <v>143</v>
       </c>
       <c r="C2" s="1" t="s">
-        <v>317</v>
+        <v>314</v>
       </c>
       <c r="D2" s="3" t="s">
         <v>23</v>
@@ -1682,14 +1681,14 @@
       </c>
     </row>
     <row r="16" spans="1:6" x14ac:dyDescent="0.3">
-      <c r="A16" s="4" t="s">
-        <v>132</v>
+      <c r="A16" s="4">
+        <v>117</v>
       </c>
       <c r="B16" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C16" s="1" t="s">
-        <v>172</v>
+        <v>179</v>
       </c>
       <c r="D16" s="3" t="s">
         <v>0</v>
@@ -1700,13 +1699,13 @@
     </row>
     <row r="17" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A17" s="4" t="s">
-        <v>49</v>
+        <v>56</v>
       </c>
       <c r="B17" s="1" t="s">
         <v>146</v>
       </c>
       <c r="C17" s="1" t="s">
-        <v>171</v>
+        <v>180</v>
       </c>
       <c r="D17" s="3" t="s">
         <v>0</v>
@@ -1716,292 +1715,292 @@
       </c>
     </row>
     <row r="18" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A18" s="4" t="s">
-        <v>42</v>
+      <c r="A18" s="4">
+        <v>147</v>
       </c>
       <c r="B18" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C18" s="1" t="s">
-        <v>173</v>
+        <v>181</v>
       </c>
       <c r="D18" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E18" s="3" t="s">
-        <v>23</v>
+        <v>9</v>
       </c>
     </row>
     <row r="19" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A19" s="4" t="s">
-        <v>43</v>
+        <v>57</v>
       </c>
       <c r="B19" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C19" s="1" t="s">
-        <v>174</v>
+        <v>182</v>
       </c>
       <c r="D19" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E19" s="3" t="s">
-        <v>0</v>
+        <v>10</v>
       </c>
     </row>
     <row r="20" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A20" s="4" t="s">
-        <v>41</v>
+        <v>135</v>
       </c>
       <c r="B20" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C20" s="1" t="s">
-        <v>175</v>
+        <v>183</v>
       </c>
       <c r="D20" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E20" s="3" t="s">
-        <v>1</v>
+        <v>11</v>
       </c>
     </row>
     <row r="21" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A21" s="4" t="s">
-        <v>50</v>
+      <c r="A21" s="4">
+        <v>132</v>
       </c>
       <c r="B21" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C21" s="1" t="s">
-        <v>187</v>
+        <v>184</v>
       </c>
       <c r="D21" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E21" s="3" t="s">
-        <v>2</v>
+        <v>12</v>
       </c>
     </row>
     <row r="22" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A22" s="4" t="s">
-        <v>51</v>
+        <v>132</v>
       </c>
       <c r="B22" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C22" s="1" t="s">
-        <v>188</v>
+        <v>172</v>
       </c>
       <c r="D22" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E22" s="3" t="s">
-        <v>3</v>
+        <v>13</v>
       </c>
     </row>
     <row r="23" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A23" s="4">
-        <v>165</v>
+      <c r="A23" s="4" t="s">
+        <v>49</v>
       </c>
       <c r="B23" s="1" t="s">
-        <v>145</v>
+        <v>146</v>
       </c>
       <c r="C23" s="1" t="s">
-        <v>176</v>
+        <v>171</v>
       </c>
       <c r="D23" s="3" t="s">
-        <v>1</v>
+        <v>0</v>
       </c>
       <c r="E23" s="3" t="s">
-        <v>4</v>
+        <v>14</v>
       </c>
     </row>
     <row r="24" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A24" s="4">
-        <v>137</v>
+      <c r="A24" s="4" t="s">
+        <v>42</v>
       </c>
       <c r="B24" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C24" s="1" t="s">
-        <v>177</v>
+        <v>173</v>
       </c>
       <c r="D24" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E24" s="3" t="s">
-        <v>5</v>
+        <v>23</v>
       </c>
     </row>
     <row r="25" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A25" s="4" t="s">
-        <v>54</v>
+        <v>43</v>
       </c>
       <c r="B25" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C25" s="1" t="s">
-        <v>178</v>
+        <v>174</v>
       </c>
       <c r="D25" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E25" s="3" t="s">
-        <v>6</v>
+        <v>0</v>
       </c>
     </row>
     <row r="26" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A26" s="4" t="s">
-        <v>55</v>
+        <v>134</v>
       </c>
       <c r="B26" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C26" s="1" t="s">
-        <v>319</v>
+        <v>318</v>
       </c>
       <c r="D26" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E26" s="3" t="s">
-        <v>7</v>
+        <v>1</v>
       </c>
     </row>
     <row r="27" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A27" s="4">
-        <v>138</v>
+      <c r="A27" s="4" t="s">
+        <v>41</v>
       </c>
       <c r="B27" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C27" s="1" t="s">
-        <v>179</v>
+        <v>175</v>
       </c>
       <c r="D27" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E27" s="3" t="s">
-        <v>8</v>
+        <v>2</v>
       </c>
     </row>
     <row r="28" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A28" s="4">
-        <v>117</v>
+      <c r="A28" s="4" t="s">
+        <v>50</v>
       </c>
       <c r="B28" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C28" s="1" t="s">
-        <v>180</v>
+        <v>185</v>
       </c>
       <c r="D28" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E28" s="3" t="s">
-        <v>9</v>
+        <v>3</v>
       </c>
     </row>
     <row r="29" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A29" s="4" t="s">
-        <v>56</v>
+        <v>51</v>
       </c>
       <c r="B29" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C29" s="1" t="s">
-        <v>181</v>
+        <v>186</v>
       </c>
       <c r="D29" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E29" s="3" t="s">
-        <v>10</v>
+        <v>4</v>
       </c>
     </row>
     <row r="30" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A30" s="4">
-        <v>147</v>
+        <v>165</v>
       </c>
       <c r="B30" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C30" s="1" t="s">
-        <v>182</v>
+        <v>176</v>
       </c>
       <c r="D30" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E30" s="3" t="s">
-        <v>11</v>
+        <v>5</v>
       </c>
     </row>
     <row r="31" spans="1:5" x14ac:dyDescent="0.3">
-      <c r="A31" s="4" t="s">
-        <v>57</v>
+      <c r="A31" s="4">
+        <v>137</v>
       </c>
       <c r="B31" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C31" s="1" t="s">
-        <v>183</v>
+        <v>177</v>
       </c>
       <c r="D31" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E31" s="3" t="s">
-        <v>12</v>
+        <v>6</v>
       </c>
     </row>
     <row r="32" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A32" s="4" t="s">
-        <v>134</v>
+        <v>54</v>
       </c>
       <c r="B32" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C32" s="1" t="s">
-        <v>184</v>
+        <v>316</v>
       </c>
       <c r="D32" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E32" s="3" t="s">
-        <v>13</v>
+        <v>7</v>
       </c>
     </row>
     <row r="33" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A33" s="4" t="s">
-        <v>135</v>
+        <v>55</v>
       </c>
       <c r="B33" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C33" s="1" t="s">
-        <v>185</v>
+        <v>317</v>
       </c>
       <c r="D33" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E33" s="3" t="s">
-        <v>14</v>
+        <v>8</v>
       </c>
     </row>
     <row r="34" spans="1:5" x14ac:dyDescent="0.3">
       <c r="A34" s="4">
-        <v>132</v>
+        <v>138</v>
       </c>
       <c r="B34" s="1" t="s">
         <v>145</v>
       </c>
       <c r="C34" s="1" t="s">
-        <v>186</v>
+        <v>178</v>
       </c>
       <c r="D34" s="3" t="s">
         <v>1</v>
       </c>
       <c r="E34" s="3" t="s">
-        <v>15</v>
+        <v>9</v>
       </c>
     </row>
     <row r="35" spans="1:5" x14ac:dyDescent="0.3">
@@ -2012,7 +2011,7 @@
         <v>150</v>
       </c>
       <c r="C35" s="1" t="s">
-        <v>221</v>
+        <v>219</v>
       </c>
       <c r="D35" s="3" t="s">
         <v>2</v>
@@ -2029,7 +2028,7 @@
         <v>150</v>
       </c>
       <c r="C36" s="1" t="s">
-        <v>222</v>
+        <v>220</v>
       </c>
       <c r="D36" s="3" t="s">
         <v>2</v>
@@ -2046,7 +2045,7 @@
         <v>150</v>
       </c>
       <c r="C37" s="1" t="s">
-        <v>223</v>
+        <v>221</v>
       </c>
       <c r="D37" s="3" t="s">
         <v>2</v>
@@ -2063,7 +2062,7 @@
         <v>150</v>
       </c>
       <c r="C38" s="1" t="s">
-        <v>224</v>
+        <v>222</v>
       </c>
       <c r="D38" s="3" t="s">
         <v>2</v>
@@ -2080,7 +2079,7 @@
         <v>150</v>
       </c>
       <c r="C39" s="1" t="s">
-        <v>225</v>
+        <v>223</v>
       </c>
       <c r="D39" s="3" t="s">
         <v>2</v>
@@ -2097,7 +2096,7 @@
         <v>150</v>
       </c>
       <c r="C40" s="1" t="s">
-        <v>226</v>
+        <v>224</v>
       </c>
       <c r="D40" s="3" t="s">
         <v>2</v>
@@ -2114,7 +2113,7 @@
         <v>150</v>
       </c>
       <c r="C41" s="1" t="s">
-        <v>227</v>
+        <v>225</v>
       </c>
       <c r="D41" s="3" t="s">
         <v>2</v>
@@ -2131,7 +2130,7 @@
         <v>150</v>
       </c>
       <c r="C42" s="1" t="s">
-        <v>228</v>
+        <v>226</v>
       </c>
       <c r="D42" s="3" t="s">
         <v>2</v>
@@ -2148,7 +2147,7 @@
         <v>150</v>
       </c>
       <c r="C43" s="1" t="s">
-        <v>229</v>
+        <v>319</v>
       </c>
       <c r="D43" s="3" t="s">
         <v>2</v>
@@ -2165,7 +2164,7 @@
         <v>150</v>
       </c>
       <c r="C44" s="1" t="s">
-        <v>230</v>
+        <v>227</v>
       </c>
       <c r="D44" s="3" t="s">
         <v>2</v>
@@ -2182,7 +2181,7 @@
         <v>150</v>
       </c>
       <c r="C45" s="1" t="s">
-        <v>231</v>
+        <v>228</v>
       </c>
       <c r="D45" s="3" t="s">
         <v>2</v>
@@ -2199,7 +2198,7 @@
         <v>150</v>
       </c>
       <c r="C46" s="1" t="s">
-        <v>232</v>
+        <v>229</v>
       </c>
       <c r="D46" s="3" t="s">
         <v>2</v>
@@ -2233,7 +2232,7 @@
         <v>150</v>
       </c>
       <c r="C48" s="1" t="s">
-        <v>233</v>
+        <v>230</v>
       </c>
       <c r="D48" s="3" t="s">
         <v>2</v>
@@ -2250,7 +2249,7 @@
         <v>150</v>
       </c>
       <c r="C49" s="1" t="s">
-        <v>234</v>
+        <v>231</v>
       </c>
       <c r="D49" s="3" t="s">
         <v>2</v>
@@ -2267,7 +2266,7 @@
         <v>150</v>
       </c>
       <c r="C50" s="1" t="s">
-        <v>235</v>
+        <v>232</v>
       </c>
       <c r="D50" s="3" t="s">
         <v>2</v>
@@ -2284,7 +2283,7 @@
         <v>150</v>
       </c>
       <c r="C51" s="1" t="s">
-        <v>236</v>
+        <v>233</v>
       </c>
       <c r="D51" s="3" t="s">
         <v>2</v>
@@ -2301,7 +2300,7 @@
         <v>150</v>
       </c>
       <c r="C52" s="1" t="s">
-        <v>237</v>
+        <v>234</v>
       </c>
       <c r="D52" s="3" t="s">
         <v>2</v>
@@ -2318,7 +2317,7 @@
         <v>150</v>
       </c>
       <c r="C53" s="1" t="s">
-        <v>238</v>
+        <v>235</v>
       </c>
       <c r="D53" s="3" t="s">
         <v>2</v>
@@ -2335,7 +2334,7 @@
         <v>150</v>
       </c>
       <c r="C54" s="1" t="s">
-        <v>239</v>
+        <v>236</v>
       </c>
       <c r="D54" s="3" t="s">
         <v>2</v>
@@ -2352,7 +2351,7 @@
         <v>150</v>
       </c>
       <c r="C55" s="1" t="s">
-        <v>240</v>
+        <v>237</v>
       </c>
       <c r="D55" s="3" t="s">
         <v>2</v>
@@ -2369,7 +2368,7 @@
         <v>150</v>
       </c>
       <c r="C56" s="1" t="s">
-        <v>241</v>
+        <v>238</v>
       </c>
       <c r="D56" s="3" t="s">
         <v>2</v>
@@ -2386,7 +2385,7 @@
         <v>150</v>
       </c>
       <c r="C57" s="1" t="s">
-        <v>242</v>
+        <v>239</v>
       </c>
       <c r="D57" s="3" t="s">
         <v>2</v>
@@ -2403,7 +2402,7 @@
         <v>150</v>
       </c>
       <c r="C58" s="1" t="s">
-        <v>243</v>
+        <v>240</v>
       </c>
       <c r="D58" s="3" t="s">
         <v>2</v>
@@ -2420,7 +2419,7 @@
         <v>150</v>
       </c>
       <c r="C59" s="1" t="s">
-        <v>244</v>
+        <v>241</v>
       </c>
       <c r="D59" s="3" t="s">
         <v>2</v>
@@ -2437,7 +2436,7 @@
         <v>150</v>
       </c>
       <c r="C60" s="1" t="s">
-        <v>245</v>
+        <v>242</v>
       </c>
       <c r="D60" s="3" t="s">
         <v>2</v>
@@ -2454,7 +2453,7 @@
         <v>150</v>
       </c>
       <c r="C61" s="1" t="s">
-        <v>246</v>
+        <v>243</v>
       </c>
       <c r="D61" s="3" t="s">
         <v>2</v>
@@ -2471,7 +2470,7 @@
         <v>150</v>
       </c>
       <c r="C62" s="1" t="s">
-        <v>247</v>
+        <v>244</v>
       </c>
       <c r="D62" s="3" t="s">
         <v>2</v>
@@ -2488,7 +2487,7 @@
         <v>150</v>
       </c>
       <c r="C63" s="1" t="s">
-        <v>248</v>
+        <v>245</v>
       </c>
       <c r="D63" s="3" t="s">
         <v>2</v>
@@ -2505,7 +2504,7 @@
         <v>150</v>
       </c>
       <c r="C64" s="1" t="s">
-        <v>249</v>
+        <v>246</v>
       </c>
       <c r="D64" s="3" t="s">
         <v>2</v>
@@ -2522,7 +2521,7 @@
         <v>150</v>
       </c>
       <c r="C65" s="1" t="s">
-        <v>250</v>
+        <v>247</v>
       </c>
       <c r="D65" s="3" t="s">
         <v>2</v>
@@ -2539,7 +2538,7 @@
         <v>147</v>
       </c>
       <c r="C66" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D66" s="3" t="s">
         <v>3</v>
@@ -2556,7 +2555,7 @@
         <v>147</v>
       </c>
       <c r="C67" s="1" t="s">
-        <v>251</v>
+        <v>248</v>
       </c>
       <c r="D67" s="3" t="s">
         <v>3</v>
@@ -2573,7 +2572,7 @@
         <v>147</v>
       </c>
       <c r="C68" s="1" t="s">
-        <v>252</v>
+        <v>249</v>
       </c>
       <c r="D68" s="3" t="s">
         <v>3</v>
@@ -2590,7 +2589,7 @@
         <v>147</v>
       </c>
       <c r="C69" s="1" t="s">
-        <v>253</v>
+        <v>250</v>
       </c>
       <c r="D69" s="3" t="s">
         <v>3</v>
@@ -2607,7 +2606,7 @@
         <v>147</v>
       </c>
       <c r="C70" s="1" t="s">
-        <v>254</v>
+        <v>251</v>
       </c>
       <c r="D70" s="3" t="s">
         <v>3</v>
@@ -2624,7 +2623,7 @@
         <v>147</v>
       </c>
       <c r="C71" s="1" t="s">
-        <v>255</v>
+        <v>252</v>
       </c>
       <c r="D71" s="3" t="s">
         <v>3</v>
@@ -2641,7 +2640,7 @@
         <v>147</v>
       </c>
       <c r="C72" s="1" t="s">
-        <v>190</v>
+        <v>188</v>
       </c>
       <c r="D72" s="3" t="s">
         <v>3</v>
@@ -2658,7 +2657,7 @@
         <v>147</v>
       </c>
       <c r="C73" s="1" t="s">
-        <v>256</v>
+        <v>253</v>
       </c>
       <c r="D73" s="3" t="s">
         <v>3</v>
@@ -2675,7 +2674,7 @@
         <v>147</v>
       </c>
       <c r="C74" s="1" t="s">
-        <v>257</v>
+        <v>254</v>
       </c>
       <c r="D74" s="3" t="s">
         <v>3</v>
@@ -2692,7 +2691,7 @@
         <v>147</v>
       </c>
       <c r="C75" s="1" t="s">
-        <v>258</v>
+        <v>255</v>
       </c>
       <c r="D75" s="3" t="s">
         <v>3</v>
@@ -2709,7 +2708,7 @@
         <v>147</v>
       </c>
       <c r="C76" s="1" t="s">
-        <v>259</v>
+        <v>256</v>
       </c>
       <c r="D76" s="3" t="s">
         <v>3</v>
@@ -2726,7 +2725,7 @@
         <v>151</v>
       </c>
       <c r="C77" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D77" s="3" t="s">
         <v>4</v>
@@ -2743,7 +2742,7 @@
         <v>151</v>
       </c>
       <c r="C78" s="1" t="s">
-        <v>260</v>
+        <v>257</v>
       </c>
       <c r="D78" s="3" t="s">
         <v>4</v>
@@ -2760,7 +2759,7 @@
         <v>151</v>
       </c>
       <c r="C79" s="1" t="s">
-        <v>261</v>
+        <v>258</v>
       </c>
       <c r="D79" s="3" t="s">
         <v>4</v>
@@ -2777,7 +2776,7 @@
         <v>151</v>
       </c>
       <c r="C80" s="1" t="s">
-        <v>262</v>
+        <v>259</v>
       </c>
       <c r="D80" s="3" t="s">
         <v>4</v>
@@ -2794,7 +2793,7 @@
         <v>151</v>
       </c>
       <c r="C81" s="1" t="s">
-        <v>263</v>
+        <v>260</v>
       </c>
       <c r="D81" s="3" t="s">
         <v>4</v>
@@ -2811,7 +2810,7 @@
         <v>152</v>
       </c>
       <c r="C82" s="1" t="s">
-        <v>264</v>
+        <v>261</v>
       </c>
       <c r="D82" s="3" t="s">
         <v>5</v>
@@ -2828,7 +2827,7 @@
         <v>152</v>
       </c>
       <c r="C83" s="1" t="s">
-        <v>265</v>
+        <v>262</v>
       </c>
       <c r="D83" s="3" t="s">
         <v>5</v>
@@ -2845,7 +2844,7 @@
         <v>152</v>
       </c>
       <c r="C84" s="1" t="s">
-        <v>266</v>
+        <v>263</v>
       </c>
       <c r="D84" s="3" t="s">
         <v>5</v>
@@ -2862,7 +2861,7 @@
         <v>152</v>
       </c>
       <c r="C85" s="1" t="s">
-        <v>267</v>
+        <v>264</v>
       </c>
       <c r="D85" s="3" t="s">
         <v>5</v>
@@ -2879,7 +2878,7 @@
         <v>152</v>
       </c>
       <c r="C86" s="1" t="s">
-        <v>268</v>
+        <v>265</v>
       </c>
       <c r="D86" s="3" t="s">
         <v>5</v>
@@ -2896,7 +2895,7 @@
         <v>152</v>
       </c>
       <c r="C87" s="1" t="s">
-        <v>269</v>
+        <v>266</v>
       </c>
       <c r="D87" s="3" t="s">
         <v>5</v>
@@ -2913,7 +2912,7 @@
         <v>152</v>
       </c>
       <c r="C88" s="1" t="s">
-        <v>270</v>
+        <v>267</v>
       </c>
       <c r="D88" s="3" t="s">
         <v>5</v>
@@ -2930,7 +2929,7 @@
         <v>152</v>
       </c>
       <c r="C89" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D89" s="3" t="s">
         <v>5</v>
@@ -2947,7 +2946,7 @@
         <v>152</v>
       </c>
       <c r="C90" s="1" t="s">
-        <v>271</v>
+        <v>268</v>
       </c>
       <c r="D90" s="3" t="s">
         <v>5</v>
@@ -2964,7 +2963,7 @@
         <v>153</v>
       </c>
       <c r="C91" s="1" t="s">
-        <v>272</v>
+        <v>269</v>
       </c>
       <c r="D91" s="3" t="s">
         <v>6</v>
@@ -2981,7 +2980,7 @@
         <v>153</v>
       </c>
       <c r="C92" s="1" t="s">
-        <v>273</v>
+        <v>270</v>
       </c>
       <c r="D92" s="3" t="s">
         <v>6</v>
@@ -2998,7 +2997,7 @@
         <v>153</v>
       </c>
       <c r="C93" s="1" t="s">
-        <v>274</v>
+        <v>271</v>
       </c>
       <c r="D93" s="3" t="s">
         <v>6</v>
@@ -3015,7 +3014,7 @@
         <v>153</v>
       </c>
       <c r="C94" s="1" t="s">
-        <v>275</v>
+        <v>272</v>
       </c>
       <c r="D94" s="3" t="s">
         <v>6</v>
@@ -3032,7 +3031,7 @@
         <v>153</v>
       </c>
       <c r="C95" s="1" t="s">
-        <v>276</v>
+        <v>273</v>
       </c>
       <c r="D95" s="3" t="s">
         <v>6</v>
@@ -3049,7 +3048,7 @@
         <v>153</v>
       </c>
       <c r="C96" s="1" t="s">
-        <v>277</v>
+        <v>274</v>
       </c>
       <c r="D96" s="3" t="s">
         <v>6</v>
@@ -3066,7 +3065,7 @@
         <v>153</v>
       </c>
       <c r="C97" s="1" t="s">
-        <v>278</v>
+        <v>275</v>
       </c>
       <c r="D97" s="3" t="s">
         <v>6</v>
@@ -3083,7 +3082,7 @@
         <v>153</v>
       </c>
       <c r="C98" s="1" t="s">
-        <v>279</v>
+        <v>276</v>
       </c>
       <c r="D98" s="3" t="s">
         <v>6</v>
@@ -3100,7 +3099,7 @@
         <v>153</v>
       </c>
       <c r="C99" s="1" t="s">
-        <v>280</v>
+        <v>277</v>
       </c>
       <c r="D99" s="3" t="s">
         <v>6</v>
@@ -3117,7 +3116,7 @@
         <v>153</v>
       </c>
       <c r="C100" s="1" t="s">
-        <v>281</v>
+        <v>278</v>
       </c>
       <c r="D100" s="3" t="s">
         <v>6</v>
@@ -3134,7 +3133,7 @@
         <v>153</v>
       </c>
       <c r="C101" s="1" t="s">
-        <v>282</v>
+        <v>279</v>
       </c>
       <c r="D101" s="3" t="s">
         <v>6</v>
@@ -3151,7 +3150,7 @@
         <v>153</v>
       </c>
       <c r="C102" s="1" t="s">
-        <v>283</v>
+        <v>280</v>
       </c>
       <c r="D102" s="3" t="s">
         <v>6</v>
@@ -3168,7 +3167,7 @@
         <v>153</v>
       </c>
       <c r="C103" s="1" t="s">
-        <v>284</v>
+        <v>281</v>
       </c>
       <c r="D103" s="3" t="s">
         <v>6</v>
@@ -3185,7 +3184,7 @@
         <v>153</v>
       </c>
       <c r="C104" s="1" t="s">
-        <v>285</v>
+        <v>282</v>
       </c>
       <c r="D104" s="3" t="s">
         <v>6</v>
@@ -3202,7 +3201,7 @@
         <v>153</v>
       </c>
       <c r="C105" s="1" t="s">
-        <v>286</v>
+        <v>283</v>
       </c>
       <c r="D105" s="3" t="s">
         <v>6</v>
@@ -3219,7 +3218,7 @@
         <v>153</v>
       </c>
       <c r="C106" s="1" t="s">
-        <v>287</v>
+        <v>284</v>
       </c>
       <c r="D106" s="3" t="s">
         <v>6</v>
@@ -3236,7 +3235,7 @@
         <v>153</v>
       </c>
       <c r="C107" s="1" t="s">
-        <v>288</v>
+        <v>285</v>
       </c>
       <c r="D107" s="3" t="s">
         <v>6</v>
@@ -3253,7 +3252,7 @@
         <v>153</v>
       </c>
       <c r="C108" s="1" t="s">
-        <v>289</v>
+        <v>286</v>
       </c>
       <c r="D108" s="3" t="s">
         <v>6</v>
@@ -3270,7 +3269,7 @@
         <v>153</v>
       </c>
       <c r="C109" s="1" t="s">
-        <v>290</v>
+        <v>287</v>
       </c>
       <c r="D109" s="3" t="s">
         <v>6</v>
@@ -3287,7 +3286,7 @@
         <v>153</v>
       </c>
       <c r="C110" s="1" t="s">
-        <v>291</v>
+        <v>288</v>
       </c>
       <c r="D110" s="3" t="s">
         <v>6</v>
@@ -3304,7 +3303,7 @@
         <v>153</v>
       </c>
       <c r="C111" s="1" t="s">
-        <v>292</v>
+        <v>289</v>
       </c>
       <c r="D111" s="3" t="s">
         <v>6</v>
@@ -3321,7 +3320,7 @@
         <v>153</v>
       </c>
       <c r="C112" s="1" t="s">
-        <v>293</v>
+        <v>290</v>
       </c>
       <c r="D112" s="3" t="s">
         <v>6</v>
@@ -3338,7 +3337,7 @@
         <v>153</v>
       </c>
       <c r="C113" s="1" t="s">
-        <v>294</v>
+        <v>291</v>
       </c>
       <c r="D113" s="3" t="s">
         <v>6</v>
@@ -3355,7 +3354,7 @@
         <v>153</v>
       </c>
       <c r="C114" s="1" t="s">
-        <v>295</v>
+        <v>292</v>
       </c>
       <c r="D114" s="3" t="s">
         <v>6</v>
@@ -3372,7 +3371,7 @@
         <v>153</v>
       </c>
       <c r="C115" s="1" t="s">
-        <v>296</v>
+        <v>293</v>
       </c>
       <c r="D115" s="3" t="s">
         <v>6</v>
@@ -3389,7 +3388,7 @@
         <v>153</v>
       </c>
       <c r="C116" s="1" t="s">
-        <v>297</v>
+        <v>294</v>
       </c>
       <c r="D116" s="3" t="s">
         <v>6</v>
@@ -3407,7 +3406,7 @@
         <v>153</v>
       </c>
       <c r="C117" s="1" t="s">
-        <v>298</v>
+        <v>295</v>
       </c>
       <c r="D117" s="3" t="s">
         <v>6</v>
@@ -3425,7 +3424,7 @@
         <v>153</v>
       </c>
       <c r="C118" s="1" t="s">
-        <v>299</v>
+        <v>296</v>
       </c>
       <c r="D118" s="3" t="s">
         <v>6</v>
@@ -3443,7 +3442,7 @@
         <v>153</v>
       </c>
       <c r="C119" s="1" t="s">
-        <v>300</v>
+        <v>297</v>
       </c>
       <c r="D119" s="3" t="s">
         <v>6</v>
@@ -3461,7 +3460,7 @@
         <v>153</v>
       </c>
       <c r="C120" s="1" t="s">
-        <v>301</v>
+        <v>298</v>
       </c>
       <c r="D120" s="3" t="s">
         <v>6</v>
@@ -3479,7 +3478,7 @@
         <v>153</v>
       </c>
       <c r="C121" s="1" t="s">
-        <v>302</v>
+        <v>299</v>
       </c>
       <c r="D121" s="3" t="s">
         <v>6</v>
@@ -3497,7 +3496,7 @@
         <v>153</v>
       </c>
       <c r="C122" s="1" t="s">
-        <v>303</v>
+        <v>300</v>
       </c>
       <c r="D122" s="3" t="s">
         <v>6</v>
@@ -3515,7 +3514,7 @@
         <v>153</v>
       </c>
       <c r="C123" s="1" t="s">
-        <v>304</v>
+        <v>301</v>
       </c>
       <c r="D123" s="3" t="s">
         <v>6</v>
@@ -3532,7 +3531,7 @@
         <v>153</v>
       </c>
       <c r="C124" s="1" t="s">
-        <v>305</v>
+        <v>302</v>
       </c>
       <c r="D124" s="3" t="s">
         <v>6</v>
@@ -3549,7 +3548,7 @@
         <v>153</v>
       </c>
       <c r="C125" s="1" t="s">
-        <v>306</v>
+        <v>303</v>
       </c>
       <c r="D125" s="3" t="s">
         <v>6</v>
@@ -3566,7 +3565,7 @@
         <v>153</v>
       </c>
       <c r="C126" s="1" t="s">
-        <v>307</v>
+        <v>304</v>
       </c>
       <c r="D126" s="3" t="s">
         <v>6</v>
@@ -3583,7 +3582,7 @@
         <v>153</v>
       </c>
       <c r="C127" s="1" t="s">
-        <v>308</v>
+        <v>305</v>
       </c>
       <c r="D127" s="3" t="s">
         <v>6</v>
@@ -3600,7 +3599,7 @@
         <v>154</v>
       </c>
       <c r="C128" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D128" s="3" t="s">
         <v>7</v>
@@ -3617,7 +3616,7 @@
         <v>154</v>
       </c>
       <c r="C129" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D129" s="3" t="s">
         <v>7</v>
@@ -3634,7 +3633,7 @@
         <v>155</v>
       </c>
       <c r="C130" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D130" s="3" t="s">
         <v>8</v>
@@ -3651,7 +3650,7 @@
         <v>155</v>
       </c>
       <c r="C131" s="1" t="s">
-        <v>310</v>
+        <v>307</v>
       </c>
       <c r="D131" s="3" t="s">
         <v>8</v>
@@ -3668,7 +3667,7 @@
         <v>155</v>
       </c>
       <c r="C132" s="1" t="s">
-        <v>311</v>
+        <v>308</v>
       </c>
       <c r="D132" s="3" t="s">
         <v>8</v>
@@ -3685,7 +3684,7 @@
         <v>155</v>
       </c>
       <c r="C133" s="1" t="s">
-        <v>312</v>
+        <v>309</v>
       </c>
       <c r="D133" s="3" t="s">
         <v>8</v>
@@ -3702,7 +3701,7 @@
         <v>155</v>
       </c>
       <c r="C134" s="1" t="s">
-        <v>313</v>
+        <v>310</v>
       </c>
       <c r="D134" s="3" t="s">
         <v>8</v>
@@ -3719,7 +3718,7 @@
         <v>155</v>
       </c>
       <c r="C135" s="1" t="s">
-        <v>314</v>
+        <v>311</v>
       </c>
       <c r="D135" s="3" t="s">
         <v>8</v>
@@ -3736,7 +3735,7 @@
         <v>155</v>
       </c>
       <c r="C136" s="1" t="s">
-        <v>315</v>
+        <v>312</v>
       </c>
       <c r="D136" s="3" t="s">
         <v>8</v>
@@ -3753,7 +3752,7 @@
         <v>155</v>
       </c>
       <c r="C137" s="1" t="s">
-        <v>316</v>
+        <v>313</v>
       </c>
       <c r="D137" s="3" t="s">
         <v>8</v>
@@ -3770,7 +3769,7 @@
         <v>155</v>
       </c>
       <c r="C138" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D138" s="3" t="s">
         <v>8</v>
@@ -3787,7 +3786,7 @@
         <v>155</v>
       </c>
       <c r="C139" s="1" t="s">
-        <v>309</v>
+        <v>306</v>
       </c>
       <c r="D139" s="3" t="s">
         <v>8</v>
@@ -3804,7 +3803,7 @@
         <v>149</v>
       </c>
       <c r="C140" s="1" t="s">
-        <v>189</v>
+        <v>187</v>
       </c>
       <c r="D140" s="3" t="s">
         <v>9</v>
@@ -3821,7 +3820,7 @@
         <v>149</v>
       </c>
       <c r="C141" s="1" t="s">
-        <v>191</v>
+        <v>189</v>
       </c>
       <c r="D141" s="3" t="s">
         <v>9</v>
@@ -3838,7 +3837,7 @@
         <v>149</v>
       </c>
       <c r="C142" s="1" t="s">
-        <v>192</v>
+        <v>190</v>
       </c>
       <c r="D142" s="3" t="s">
         <v>9</v>
@@ -3855,7 +3854,7 @@
         <v>149</v>
       </c>
       <c r="C143" s="1" t="s">
-        <v>193</v>
+        <v>191</v>
       </c>
       <c r="D143" s="3" t="s">
         <v>9</v>
@@ -3872,7 +3871,7 @@
         <v>149</v>
       </c>
       <c r="C144" s="1" t="s">
-        <v>194</v>
+        <v>192</v>
       </c>
       <c r="D144" s="3" t="s">
         <v>9</v>
@@ -3889,7 +3888,7 @@
         <v>149</v>
       </c>
       <c r="C145" s="1" t="s">
-        <v>195</v>
+        <v>193</v>
       </c>
       <c r="D145" s="3" t="s">
         <v>9</v>
@@ -3906,7 +3905,7 @@
         <v>149</v>
       </c>
       <c r="C146" s="1" t="s">
-        <v>196</v>
+        <v>194</v>
       </c>
       <c r="D146" s="3" t="s">
         <v>9</v>
@@ -3923,7 +3922,7 @@
         <v>149</v>
       </c>
       <c r="C147" s="1" t="s">
-        <v>197</v>
+        <v>195</v>
       </c>
       <c r="D147" s="3" t="s">
         <v>9</v>
@@ -3940,7 +3939,7 @@
         <v>149</v>
       </c>
       <c r="C148" s="1" t="s">
-        <v>198</v>
+        <v>196</v>
       </c>
       <c r="D148" s="3" t="s">
         <v>9</v>
@@ -3957,7 +3956,7 @@
         <v>149</v>
       </c>
       <c r="C149" s="1" t="s">
-        <v>199</v>
+        <v>197</v>
       </c>
       <c r="D149" s="3" t="s">
         <v>9</v>
@@ -3974,7 +3973,7 @@
         <v>149</v>
       </c>
       <c r="C150" s="1" t="s">
-        <v>200</v>
+        <v>198</v>
       </c>
       <c r="D150" s="3" t="s">
         <v>9</v>
@@ -3991,7 +3990,7 @@
         <v>149</v>
       </c>
       <c r="C151" s="1" t="s">
-        <v>201</v>
+        <v>199</v>
       </c>
       <c r="D151" s="3" t="s">
         <v>9</v>
@@ -4008,7 +4007,7 @@
         <v>149</v>
       </c>
       <c r="C152" s="1" t="s">
-        <v>202</v>
+        <v>200</v>
       </c>
       <c r="D152" s="3" t="s">
         <v>9</v>
@@ -4025,7 +4024,7 @@
         <v>149</v>
       </c>
       <c r="C153" s="1" t="s">
-        <v>203</v>
+        <v>201</v>
       </c>
       <c r="D153" s="3" t="s">
         <v>9</v>
@@ -4042,7 +4041,7 @@
         <v>149</v>
       </c>
       <c r="C154" s="1" t="s">
-        <v>204</v>
+        <v>202</v>
       </c>
       <c r="D154" s="3" t="s">
         <v>9</v>
@@ -4059,7 +4058,7 @@
         <v>149</v>
       </c>
       <c r="C155" s="1" t="s">
-        <v>205</v>
+        <v>203</v>
       </c>
       <c r="D155" s="3" t="s">
         <v>9</v>
@@ -4076,7 +4075,7 @@
         <v>156</v>
       </c>
       <c r="C156" s="1" t="s">
-        <v>212</v>
+        <v>210</v>
       </c>
       <c r="D156" s="3" t="s">
         <v>10</v>
@@ -4093,7 +4092,7 @@
         <v>156</v>
       </c>
       <c r="C157" s="1" t="s">
-        <v>213</v>
+        <v>211</v>
       </c>
       <c r="D157" s="3" t="s">
         <v>10</v>
@@ -4110,7 +4109,7 @@
         <v>156</v>
       </c>
       <c r="C158" s="1" t="s">
-        <v>214</v>
+        <v>212</v>
       </c>
       <c r="D158" s="3" t="s">
         <v>10</v>
@@ -4127,7 +4126,7 @@
         <v>156</v>
       </c>
       <c r="C159" s="1" t="s">
-        <v>215</v>
+        <v>213</v>
       </c>
       <c r="D159" s="3" t="s">
         <v>10</v>
@@ -4144,7 +4143,7 @@
         <v>156</v>
       </c>
       <c r="C160" s="1" t="s">
-        <v>216</v>
+        <v>214</v>
       </c>
       <c r="D160" s="3" t="s">
         <v>10</v>
@@ -4161,7 +4160,7 @@
         <v>156</v>
       </c>
       <c r="C161" s="1" t="s">
-        <v>217</v>
+        <v>215</v>
       </c>
       <c r="D161" s="3" t="s">
         <v>10</v>
@@ -4178,7 +4177,7 @@
         <v>156</v>
       </c>
       <c r="C162" s="1" t="s">
-        <v>218</v>
+        <v>216</v>
       </c>
       <c r="D162" s="3" t="s">
         <v>10</v>
@@ -4195,7 +4194,7 @@
         <v>156</v>
       </c>
       <c r="C163" s="1" t="s">
-        <v>219</v>
+        <v>217</v>
       </c>
       <c r="D163" s="3" t="s">
         <v>10</v>
@@ -4212,7 +4211,7 @@
         <v>156</v>
       </c>
       <c r="C164" s="1" t="s">
-        <v>220</v>
+        <v>218</v>
       </c>
       <c r="D164" s="3" t="s">
         <v>10</v>
@@ -4229,7 +4228,7 @@
         <v>148</v>
       </c>
       <c r="C165" s="1" t="s">
-        <v>206</v>
+        <v>204</v>
       </c>
       <c r="D165" s="3" t="s">
         <v>11</v>
@@ -4246,7 +4245,7 @@
         <v>148</v>
       </c>
       <c r="C166" s="1" t="s">
-        <v>207</v>
+        <v>205</v>
       </c>
       <c r="D166" s="3" t="s">
         <v>11</v>
@@ -4263,7 +4262,7 @@
         <v>148</v>
       </c>
       <c r="C167" s="1" t="s">
-        <v>208</v>
+        <v>206</v>
       </c>
       <c r="D167" s="3" t="s">
         <v>11</v>
@@ -4280,7 +4279,7 @@
         <v>148</v>
       </c>
       <c r="C168" s="1" t="s">
-        <v>210</v>
+        <v>208</v>
       </c>
       <c r="D168" s="3" t="s">
         <v>11</v>
@@ -4297,7 +4296,7 @@
         <v>148</v>
       </c>
       <c r="C169" s="1" t="s">
-        <v>209</v>
+        <v>207</v>
       </c>
       <c r="D169" s="3" t="s">
         <v>11</v>
@@ -4314,7 +4313,7 @@
         <v>148</v>
       </c>
       <c r="C170" s="1" t="s">
-        <v>211</v>
+        <v>209</v>
       </c>
       <c r="D170" s="3" t="s">
         <v>11</v>
@@ -4328,7 +4327,7 @@
         <v>171</v>
       </c>
       <c r="B171" s="1" t="s">
-        <v>318</v>
+        <v>315</v>
       </c>
       <c r="C171" s="1" t="s">
         <v>144</v>

</xml_diff>